<commit_message>
Risk Suggestions at part-supplier combo level
Each row is now a combo: part label + Supplier + Process/part type
dropdowns; performance averages and the Quality_Compliance / Capacity
suggestions filter to that supplier's projects of that process (blank
process = all their projects). Supplier_Stability stays supplier-wide by
design - stability is about the supplier as a business, with Cost and
Responsiveness as its evidence.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CFoRmmyZBAk7VkisRgH6G2
</commit_message>
<xml_diff>
--- a/Part-Supplier Risk Model/Supplier_Scorecard.xlsx
+++ b/Part-Supplier Risk Model/Supplier_Scorecard.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="151">
   <si>
     <t xml:space="preserve">Supplier Scorecard — how to use</t>
   </si>
@@ -258,18 +258,24 @@
     <t xml:space="preserve">Risk Suggestions - feed for the Part-Supplier Risk Model</t>
   </si>
   <si>
-    <t xml:space="preserve">Fully automatic, one row per supplier. Translation: risk = 6 - average performance (scorecard 5 = excellent -&gt; risk 1 = low), rounded to the nearest whole score and clamped to 1-5. Type the suggested values into the PART_RISK tab of Part_Supplier_Risk_Model - they are a starting point, not an override; adjust with judgment and with what the scorecard cannot see.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUPPLIER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCORECARD PERFORMANCE (auto, 5 = excellent)</t>
+    <t xml:space="preserve">One row per PART-SUPPLIER combo: label the part (as it will appear in PART_RISK), pick the Supplier and the Process/part type that makes it - the averages then use only that supplier's logged projects of that process. Leave Process blank to use all the supplier's projects. Translation: risk = 6 - average performance (scorecard 5 = excellent -&gt; risk 1 = low), rounded and clamped to 1-5. Type the suggested values into the PART_RISK tab of Part_Supplier_Risk_Model - a starting point, not an override.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. LABEL THE PART</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. PICK THE COMBO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCORECARD PERFORMANCE FOR THE COMBO (auto, 5 = excellent)</t>
   </si>
   <si>
     <t xml:space="preserve">SUGGESTED RISK ENTRIES FOR PART_RISK (1 = low risk ... 5 = high)</t>
   </si>
   <si>
+    <t xml:space="preserve">Part (number / description)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Quality_Compliance (suggest)</t>
   </si>
   <si>
@@ -279,22 +285,28 @@
     <t xml:space="preserve">Supplier_Stability (suggest)</t>
   </si>
   <si>
+    <t xml:space="preserve">cA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rA</t>
+  </si>
+  <si>
     <t xml:space="preserve">HOW THE TRANSLATION WORKS</t>
   </si>
   <si>
-    <t xml:space="preserve">Quality_Compliance  &lt;-  6 - avg Quality.  What they actually delivered is direct evidence for the part's quality risk.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capacity  &lt;-  6 - avg Lead time.  Observed delivery performance is the visible side of capacity; sanity-check against On-time %.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supplier_Stability  &lt;-  6 - average(Responsiveness, Cost).  Cost has no part-level column in the risk register, but erratic pricing and poor cost transparency - like slow communication - are evidence about the supplier as a business, so both feed the Stability suggestion.</t>
+    <t xml:space="preserve">Quality_Compliance  &lt;-  6 - avg Quality of THIS combo (this supplier's projects of this process).  What they delivered on this kind of part is direct evidence for its quality risk.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacity  &lt;-  6 - avg Lead time of THIS combo.  Observed delivery performance is the visible side of capacity; sanity-check against On-time %.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supplier_Stability  &lt;-  6 - average(Responsiveness, Cost) across ALL the supplier's projects, regardless of process - stability is about the supplier as a business, not one part. Cost has no part-level column in the risk register, but erratic pricing and poor cost transparency - like slow communication - are stability evidence.</t>
   </si>
   <si>
     <t xml:space="preserve">No scorecard equivalent - score these by judgment in the master model:  Sourcing_Backup (do alternatives exist?),  External_Factors (location, logistics, borders),  Impact (what the part means to the model),  Qty_per_Model / volume.</t>
   </si>
   <si>
-    <t xml:space="preserve">Suggestions round to the nearest whole score and clamp to 1-5. A supplier with few projects logged (see Projects column) is thin evidence - weigh it accordingly.</t>
+    <t xml:space="preserve">Suggestions round to the nearest whole score and clamp to 1-5. Few projects behind a combo (see Projects column) = thin evidence - weigh it accordingly.</t>
   </si>
   <si>
     <t xml:space="preserve">Supplier directory</t>
@@ -478,7 +490,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="166" formatCode="0"/>
@@ -486,8 +498,7 @@
     <numFmt numFmtId="168" formatCode="#,##0"/>
     <numFmt numFmtId="169" formatCode="0.0%"/>
     <numFmt numFmtId="170" formatCode="0%"/>
-    <numFmt numFmtId="171" formatCode="General"/>
-    <numFmt numFmtId="172" formatCode="0.0"/>
+    <numFmt numFmtId="171" formatCode="0.0"/>
   </numFmts>
   <fonts count="25">
     <font>
@@ -672,7 +683,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -705,8 +716,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFF6DC"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFFFF6DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -925,15 +942,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -941,7 +958,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="19" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -981,11 +998,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="24" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="24" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1142,7 +1159,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF2CC"/>
+      <rgbColor rgb="FFFFF6DC"/>
       <rgbColor rgb="FFF2F2F2"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFF8696B"/>
@@ -1159,7 +1176,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFD9E2F3"/>
       <rgbColor rgb="FFF9F9F9"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFF2CC"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -1353,11 +1370,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="29834272"/>
-        <c:axId val="67701022"/>
+        <c:axId val="68840439"/>
+        <c:axId val="82587896"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="29834272"/>
+        <c:axId val="68840439"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1389,7 +1406,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67701022"/>
+        <c:crossAx val="82587896"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1397,7 +1414,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="67701022"/>
+        <c:axId val="82587896"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="5"/>
@@ -1441,7 +1458,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29834272"/>
+        <c:crossAx val="68840439"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -11721,18 +11738,22 @@
     <tabColor rgb="FFC00000"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:P52"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="16" min="15" style="0" width="4"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11753,1523 +11774,2290 @@
         <v>77</v>
       </c>
       <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
+      <c r="D3" s="35" t="s">
+        <v>78</v>
+      </c>
       <c r="E3" s="35"/>
       <c r="F3" s="35"/>
       <c r="G3" s="35"/>
       <c r="H3" s="35"/>
-      <c r="I3" s="35" t="s">
-        <v>78</v>
-      </c>
+      <c r="I3" s="35"/>
       <c r="J3" s="35"/>
-      <c r="K3" s="35"/>
+      <c r="K3" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="C4" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="E4" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="F4" s="36" t="s">
         <v>65</v>
       </c>
-      <c r="E4" s="36" t="s">
+      <c r="G4" s="36" t="s">
         <v>66</v>
       </c>
-      <c r="F4" s="36" t="s">
+      <c r="H4" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="G4" s="36" t="s">
+      <c r="I4" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="H4" s="36" t="s">
+      <c r="J4" s="36" t="s">
         <v>69</v>
-      </c>
-      <c r="I4" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="J4" s="36" t="s">
-        <v>80</v>
       </c>
       <c r="K4" s="36" t="s">
         <v>81</v>
       </c>
+      <c r="L4" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="M4" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="O4" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="P4" s="33" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="37" t="str">
-        <f aca="false">IF(Suppliers!A3="","",Suppliers!A3)</f>
-        <v>Fictiv</v>
-      </c>
-      <c r="B5" s="38" t="n">
-        <f aca="false">IF($A5="","",COUNTIF('Score Log'!$C$4:$C$203,$A5))</f>
-        <v>1</v>
-      </c>
-      <c r="C5" s="39" t="n">
-        <f aca="false">IF($A5="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A5),1),"-"))</f>
-        <v>4</v>
-      </c>
-      <c r="D5" s="39" t="n">
-        <f aca="false">IF($A5="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A5),1),"-"))</f>
-        <v>5</v>
-      </c>
-      <c r="E5" s="39" t="n">
-        <f aca="false">IF($A5="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A5),1),"-"))</f>
-        <v>4</v>
-      </c>
-      <c r="F5" s="39" t="n">
-        <f aca="false">IF($A5="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A5),1),"-"))</f>
-        <v>5</v>
-      </c>
-      <c r="G5" s="39" t="n">
-        <f aca="false">IF($A5="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A5),1),"-"))</f>
-        <v>4.5</v>
-      </c>
-      <c r="H5" s="40" t="n">
-        <f aca="false">IF($A5="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A5,'Score Log'!$U$4:$U$203,"Yes")/$B5,"-"))</f>
-        <v>1</v>
-      </c>
-      <c r="I5" s="41" t="n">
-        <f aca="false">IF($A5="","",IF(ISNUMBER($D5),MAX(1,MIN(5,ROUND(6-$D5,0))),"-"))</f>
-        <v>1</v>
-      </c>
-      <c r="J5" s="41" t="n">
-        <f aca="false">IF($A5="","",IF(ISNUMBER($E5),MAX(1,MIN(5,ROUND(6-$E5,0))),"-"))</f>
-        <v>2</v>
-      </c>
-      <c r="K5" s="41" t="n">
-        <f aca="false">IF($A5="","",IF(AND(ISNUMBER($F5),ISNUMBER($C5)),MAX(1,MIN(5,ROUND(6-AVERAGE($F5,$C5),0))),IF(ISNUMBER($F5),MAX(1,MIN(5,ROUND(6-$F5,0))),"-")))</f>
-        <v>2</v>
+      <c r="A5" s="37"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="38" t="str">
+        <f aca="false">IF($B5="","",IF($C5="",COUNTIF('Score Log'!$C$4:$C$203,$B5),COUNTIFS('Score Log'!$C$4:$C$203,$B5,'Score Log'!$D$4:$D$203,$C5)))</f>
+        <v/>
+      </c>
+      <c r="E5" s="39" t="str">
+        <f aca="false">IF($B5="","",IFERROR(ROUND(IF($C5="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B5),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B5,'Score Log'!$D$4:$D$203,$C5)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="F5" s="39" t="str">
+        <f aca="false">IF($B5="","",IFERROR(ROUND(IF($C5="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B5),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B5,'Score Log'!$D$4:$D$203,$C5)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="G5" s="39" t="str">
+        <f aca="false">IF($B5="","",IFERROR(ROUND(IF($C5="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B5),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B5,'Score Log'!$D$4:$D$203,$C5)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H5" s="39" t="str">
+        <f aca="false">IF($B5="","",IFERROR(ROUND(IF($C5="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B5),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B5,'Score Log'!$D$4:$D$203,$C5)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I5" s="39" t="str">
+        <f aca="false">IF($B5="","",IFERROR(ROUND(IF($C5="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B5),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B5,'Score Log'!$D$4:$D$203,$C5)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J5" s="40" t="str">
+        <f aca="false">IF(OR($B5="",$D5=0),"",IFERROR(IF($C5="",COUNTIFS('Score Log'!$C$4:$C$203,$B5,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B5,'Score Log'!$D$4:$D$203,$C5,'Score Log'!$U$4:$U$203,"Yes"))/$D5,"-"))</f>
+        <v/>
+      </c>
+      <c r="K5" s="41" t="str">
+        <f aca="false">IF($B5="","",IF(ISNUMBER($F5),MAX(1,MIN(5,ROUND(6-$F5,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L5" s="41" t="str">
+        <f aca="false">IF($B5="","",IF(ISNUMBER($G5),MAX(1,MIN(5,ROUND(6-$G5,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M5" s="41" t="str">
+        <f aca="false">IF($B5="","",IF(AND(ISNUMBER($P5),ISNUMBER($O5)),MAX(1,MIN(5,ROUND(6-AVERAGE($P5,$O5),0))),IF(ISNUMBER($P5),MAX(1,MIN(5,ROUND(6-$P5,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O5" s="33" t="str">
+        <f aca="false">IF($B5="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B5),""))</f>
+        <v/>
+      </c>
+      <c r="P5" s="33" t="str">
+        <f aca="false">IF($B5="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B5),""))</f>
+        <v/>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="37" t="str">
-        <f aca="false">IF(Suppliers!A4="","",Suppliers!A4)</f>
-        <v>Advanced Plastiform</v>
-      </c>
-      <c r="B6" s="38" t="n">
-        <f aca="false">IF($A6="","",COUNTIF('Score Log'!$C$4:$C$203,$A6))</f>
-        <v>1</v>
-      </c>
-      <c r="C6" s="39" t="str">
-        <f aca="false">IF($A6="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A6),1),"-"))</f>
-        <v>-</v>
-      </c>
-      <c r="D6" s="39" t="str">
-        <f aca="false">IF($A6="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A6),1),"-"))</f>
-        <v>-</v>
+      <c r="A6" s="37"/>
+      <c r="B6" s="37"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="38" t="str">
+        <f aca="false">IF($B6="","",IF($C6="",COUNTIF('Score Log'!$C$4:$C$203,$B6),COUNTIFS('Score Log'!$C$4:$C$203,$B6,'Score Log'!$D$4:$D$203,$C6)))</f>
+        <v/>
       </c>
       <c r="E6" s="39" t="str">
-        <f aca="false">IF($A6="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A6),1),"-"))</f>
-        <v>-</v>
+        <f aca="false">IF($B6="","",IFERROR(ROUND(IF($C6="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B6),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B6,'Score Log'!$D$4:$D$203,$C6)),1),"-"))</f>
+        <v/>
       </c>
       <c r="F6" s="39" t="str">
-        <f aca="false">IF($A6="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A6),1),"-"))</f>
-        <v>-</v>
+        <f aca="false">IF($B6="","",IFERROR(ROUND(IF($C6="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B6),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B6,'Score Log'!$D$4:$D$203,$C6)),1),"-"))</f>
+        <v/>
       </c>
       <c r="G6" s="39" t="str">
-        <f aca="false">IF($A6="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A6),1),"-"))</f>
-        <v>-</v>
-      </c>
-      <c r="H6" s="40" t="n">
-        <f aca="false">IF($A6="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A6,'Score Log'!$U$4:$U$203,"Yes")/$B6,"-"))</f>
-        <v>0</v>
-      </c>
-      <c r="I6" s="41" t="str">
-        <f aca="false">IF($A6="","",IF(ISNUMBER($D6),MAX(1,MIN(5,ROUND(6-$D6,0))),"-"))</f>
-        <v>-</v>
-      </c>
-      <c r="J6" s="41" t="str">
-        <f aca="false">IF($A6="","",IF(ISNUMBER($E6),MAX(1,MIN(5,ROUND(6-$E6,0))),"-"))</f>
-        <v>-</v>
+        <f aca="false">IF($B6="","",IFERROR(ROUND(IF($C6="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B6),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B6,'Score Log'!$D$4:$D$203,$C6)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H6" s="39" t="str">
+        <f aca="false">IF($B6="","",IFERROR(ROUND(IF($C6="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B6),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B6,'Score Log'!$D$4:$D$203,$C6)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I6" s="39" t="str">
+        <f aca="false">IF($B6="","",IFERROR(ROUND(IF($C6="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B6),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B6,'Score Log'!$D$4:$D$203,$C6)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J6" s="40" t="str">
+        <f aca="false">IF(OR($B6="",$D6=0),"",IFERROR(IF($C6="",COUNTIFS('Score Log'!$C$4:$C$203,$B6,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B6,'Score Log'!$D$4:$D$203,$C6,'Score Log'!$U$4:$U$203,"Yes"))/$D6,"-"))</f>
+        <v/>
       </c>
       <c r="K6" s="41" t="str">
-        <f aca="false">IF($A6="","",IF(AND(ISNUMBER($F6),ISNUMBER($C6)),MAX(1,MIN(5,ROUND(6-AVERAGE($F6,$C6),0))),IF(ISNUMBER($F6),MAX(1,MIN(5,ROUND(6-$F6,0))),"-")))</f>
-        <v>-</v>
+        <f aca="false">IF($B6="","",IF(ISNUMBER($F6),MAX(1,MIN(5,ROUND(6-$F6,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L6" s="41" t="str">
+        <f aca="false">IF($B6="","",IF(ISNUMBER($G6),MAX(1,MIN(5,ROUND(6-$G6,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M6" s="41" t="str">
+        <f aca="false">IF($B6="","",IF(AND(ISNUMBER($P6),ISNUMBER($O6)),MAX(1,MIN(5,ROUND(6-AVERAGE($P6,$O6),0))),IF(ISNUMBER($P6),MAX(1,MIN(5,ROUND(6-$P6,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O6" s="33" t="str">
+        <f aca="false">IF($B6="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B6),""))</f>
+        <v/>
+      </c>
+      <c r="P6" s="33" t="str">
+        <f aca="false">IF($B6="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B6),""))</f>
+        <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="37" t="str">
-        <f aca="false">IF(Suppliers!A5="","",Suppliers!A5)</f>
-        <v/>
-      </c>
-      <c r="B7" s="38" t="str">
-        <f aca="false">IF($A7="","",COUNTIF('Score Log'!$C$4:$C$203,$A7))</f>
-        <v/>
-      </c>
-      <c r="C7" s="39" t="str">
-        <f aca="false">IF($A7="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A7),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D7" s="39" t="str">
-        <f aca="false">IF($A7="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A7),1),"-"))</f>
+      <c r="A7" s="37"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="38" t="str">
+        <f aca="false">IF($B7="","",IF($C7="",COUNTIF('Score Log'!$C$4:$C$203,$B7),COUNTIFS('Score Log'!$C$4:$C$203,$B7,'Score Log'!$D$4:$D$203,$C7)))</f>
         <v/>
       </c>
       <c r="E7" s="39" t="str">
-        <f aca="false">IF($A7="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A7),1),"-"))</f>
+        <f aca="false">IF($B7="","",IFERROR(ROUND(IF($C7="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B7),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B7,'Score Log'!$D$4:$D$203,$C7)),1),"-"))</f>
         <v/>
       </c>
       <c r="F7" s="39" t="str">
-        <f aca="false">IF($A7="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A7),1),"-"))</f>
+        <f aca="false">IF($B7="","",IFERROR(ROUND(IF($C7="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B7),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B7,'Score Log'!$D$4:$D$203,$C7)),1),"-"))</f>
         <v/>
       </c>
       <c r="G7" s="39" t="str">
-        <f aca="false">IF($A7="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A7),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H7" s="40" t="str">
-        <f aca="false">IF($A7="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A7,'Score Log'!$U$4:$U$203,"Yes")/$B7,"-"))</f>
-        <v/>
-      </c>
-      <c r="I7" s="41" t="str">
-        <f aca="false">IF($A7="","",IF(ISNUMBER($D7),MAX(1,MIN(5,ROUND(6-$D7,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J7" s="41" t="str">
-        <f aca="false">IF($A7="","",IF(ISNUMBER($E7),MAX(1,MIN(5,ROUND(6-$E7,0))),"-"))</f>
+        <f aca="false">IF($B7="","",IFERROR(ROUND(IF($C7="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B7),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B7,'Score Log'!$D$4:$D$203,$C7)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H7" s="39" t="str">
+        <f aca="false">IF($B7="","",IFERROR(ROUND(IF($C7="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B7),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B7,'Score Log'!$D$4:$D$203,$C7)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I7" s="39" t="str">
+        <f aca="false">IF($B7="","",IFERROR(ROUND(IF($C7="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B7),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B7,'Score Log'!$D$4:$D$203,$C7)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J7" s="40" t="str">
+        <f aca="false">IF(OR($B7="",$D7=0),"",IFERROR(IF($C7="",COUNTIFS('Score Log'!$C$4:$C$203,$B7,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B7,'Score Log'!$D$4:$D$203,$C7,'Score Log'!$U$4:$U$203,"Yes"))/$D7,"-"))</f>
         <v/>
       </c>
       <c r="K7" s="41" t="str">
-        <f aca="false">IF($A7="","",IF(AND(ISNUMBER($F7),ISNUMBER($C7)),MAX(1,MIN(5,ROUND(6-AVERAGE($F7,$C7),0))),IF(ISNUMBER($F7),MAX(1,MIN(5,ROUND(6-$F7,0))),"-")))</f>
+        <f aca="false">IF($B7="","",IF(ISNUMBER($F7),MAX(1,MIN(5,ROUND(6-$F7,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L7" s="41" t="str">
+        <f aca="false">IF($B7="","",IF(ISNUMBER($G7),MAX(1,MIN(5,ROUND(6-$G7,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M7" s="41" t="str">
+        <f aca="false">IF($B7="","",IF(AND(ISNUMBER($P7),ISNUMBER($O7)),MAX(1,MIN(5,ROUND(6-AVERAGE($P7,$O7),0))),IF(ISNUMBER($P7),MAX(1,MIN(5,ROUND(6-$P7,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O7" s="33" t="str">
+        <f aca="false">IF($B7="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B7),""))</f>
+        <v/>
+      </c>
+      <c r="P7" s="33" t="str">
+        <f aca="false">IF($B7="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B7),""))</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="37" t="str">
-        <f aca="false">IF(Suppliers!A6="","",Suppliers!A6)</f>
-        <v/>
-      </c>
-      <c r="B8" s="38" t="str">
-        <f aca="false">IF($A8="","",COUNTIF('Score Log'!$C$4:$C$203,$A8))</f>
-        <v/>
-      </c>
-      <c r="C8" s="39" t="str">
-        <f aca="false">IF($A8="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A8),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D8" s="39" t="str">
-        <f aca="false">IF($A8="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A8),1),"-"))</f>
+      <c r="A8" s="37"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="38" t="str">
+        <f aca="false">IF($B8="","",IF($C8="",COUNTIF('Score Log'!$C$4:$C$203,$B8),COUNTIFS('Score Log'!$C$4:$C$203,$B8,'Score Log'!$D$4:$D$203,$C8)))</f>
         <v/>
       </c>
       <c r="E8" s="39" t="str">
-        <f aca="false">IF($A8="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A8),1),"-"))</f>
+        <f aca="false">IF($B8="","",IFERROR(ROUND(IF($C8="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B8),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B8,'Score Log'!$D$4:$D$203,$C8)),1),"-"))</f>
         <v/>
       </c>
       <c r="F8" s="39" t="str">
-        <f aca="false">IF($A8="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A8),1),"-"))</f>
+        <f aca="false">IF($B8="","",IFERROR(ROUND(IF($C8="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B8),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B8,'Score Log'!$D$4:$D$203,$C8)),1),"-"))</f>
         <v/>
       </c>
       <c r="G8" s="39" t="str">
-        <f aca="false">IF($A8="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A8),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H8" s="40" t="str">
-        <f aca="false">IF($A8="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A8,'Score Log'!$U$4:$U$203,"Yes")/$B8,"-"))</f>
-        <v/>
-      </c>
-      <c r="I8" s="41" t="str">
-        <f aca="false">IF($A8="","",IF(ISNUMBER($D8),MAX(1,MIN(5,ROUND(6-$D8,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J8" s="41" t="str">
-        <f aca="false">IF($A8="","",IF(ISNUMBER($E8),MAX(1,MIN(5,ROUND(6-$E8,0))),"-"))</f>
+        <f aca="false">IF($B8="","",IFERROR(ROUND(IF($C8="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B8),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B8,'Score Log'!$D$4:$D$203,$C8)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H8" s="39" t="str">
+        <f aca="false">IF($B8="","",IFERROR(ROUND(IF($C8="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B8),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B8,'Score Log'!$D$4:$D$203,$C8)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I8" s="39" t="str">
+        <f aca="false">IF($B8="","",IFERROR(ROUND(IF($C8="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B8),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B8,'Score Log'!$D$4:$D$203,$C8)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J8" s="40" t="str">
+        <f aca="false">IF(OR($B8="",$D8=0),"",IFERROR(IF($C8="",COUNTIFS('Score Log'!$C$4:$C$203,$B8,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B8,'Score Log'!$D$4:$D$203,$C8,'Score Log'!$U$4:$U$203,"Yes"))/$D8,"-"))</f>
         <v/>
       </c>
       <c r="K8" s="41" t="str">
-        <f aca="false">IF($A8="","",IF(AND(ISNUMBER($F8),ISNUMBER($C8)),MAX(1,MIN(5,ROUND(6-AVERAGE($F8,$C8),0))),IF(ISNUMBER($F8),MAX(1,MIN(5,ROUND(6-$F8,0))),"-")))</f>
+        <f aca="false">IF($B8="","",IF(ISNUMBER($F8),MAX(1,MIN(5,ROUND(6-$F8,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L8" s="41" t="str">
+        <f aca="false">IF($B8="","",IF(ISNUMBER($G8),MAX(1,MIN(5,ROUND(6-$G8,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M8" s="41" t="str">
+        <f aca="false">IF($B8="","",IF(AND(ISNUMBER($P8),ISNUMBER($O8)),MAX(1,MIN(5,ROUND(6-AVERAGE($P8,$O8),0))),IF(ISNUMBER($P8),MAX(1,MIN(5,ROUND(6-$P8,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O8" s="33" t="str">
+        <f aca="false">IF($B8="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B8),""))</f>
+        <v/>
+      </c>
+      <c r="P8" s="33" t="str">
+        <f aca="false">IF($B8="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B8),""))</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="37" t="str">
-        <f aca="false">IF(Suppliers!A7="","",Suppliers!A7)</f>
-        <v/>
-      </c>
-      <c r="B9" s="38" t="str">
-        <f aca="false">IF($A9="","",COUNTIF('Score Log'!$C$4:$C$203,$A9))</f>
-        <v/>
-      </c>
-      <c r="C9" s="39" t="str">
-        <f aca="false">IF($A9="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A9),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D9" s="39" t="str">
-        <f aca="false">IF($A9="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A9),1),"-"))</f>
+      <c r="A9" s="37"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="38" t="str">
+        <f aca="false">IF($B9="","",IF($C9="",COUNTIF('Score Log'!$C$4:$C$203,$B9),COUNTIFS('Score Log'!$C$4:$C$203,$B9,'Score Log'!$D$4:$D$203,$C9)))</f>
         <v/>
       </c>
       <c r="E9" s="39" t="str">
-        <f aca="false">IF($A9="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A9),1),"-"))</f>
+        <f aca="false">IF($B9="","",IFERROR(ROUND(IF($C9="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B9),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B9,'Score Log'!$D$4:$D$203,$C9)),1),"-"))</f>
         <v/>
       </c>
       <c r="F9" s="39" t="str">
-        <f aca="false">IF($A9="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A9),1),"-"))</f>
+        <f aca="false">IF($B9="","",IFERROR(ROUND(IF($C9="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B9),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B9,'Score Log'!$D$4:$D$203,$C9)),1),"-"))</f>
         <v/>
       </c>
       <c r="G9" s="39" t="str">
-        <f aca="false">IF($A9="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A9),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H9" s="40" t="str">
-        <f aca="false">IF($A9="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A9,'Score Log'!$U$4:$U$203,"Yes")/$B9,"-"))</f>
-        <v/>
-      </c>
-      <c r="I9" s="41" t="str">
-        <f aca="false">IF($A9="","",IF(ISNUMBER($D9),MAX(1,MIN(5,ROUND(6-$D9,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J9" s="41" t="str">
-        <f aca="false">IF($A9="","",IF(ISNUMBER($E9),MAX(1,MIN(5,ROUND(6-$E9,0))),"-"))</f>
+        <f aca="false">IF($B9="","",IFERROR(ROUND(IF($C9="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B9),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B9,'Score Log'!$D$4:$D$203,$C9)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H9" s="39" t="str">
+        <f aca="false">IF($B9="","",IFERROR(ROUND(IF($C9="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B9),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B9,'Score Log'!$D$4:$D$203,$C9)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I9" s="39" t="str">
+        <f aca="false">IF($B9="","",IFERROR(ROUND(IF($C9="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B9),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B9,'Score Log'!$D$4:$D$203,$C9)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J9" s="40" t="str">
+        <f aca="false">IF(OR($B9="",$D9=0),"",IFERROR(IF($C9="",COUNTIFS('Score Log'!$C$4:$C$203,$B9,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B9,'Score Log'!$D$4:$D$203,$C9,'Score Log'!$U$4:$U$203,"Yes"))/$D9,"-"))</f>
         <v/>
       </c>
       <c r="K9" s="41" t="str">
-        <f aca="false">IF($A9="","",IF(AND(ISNUMBER($F9),ISNUMBER($C9)),MAX(1,MIN(5,ROUND(6-AVERAGE($F9,$C9),0))),IF(ISNUMBER($F9),MAX(1,MIN(5,ROUND(6-$F9,0))),"-")))</f>
+        <f aca="false">IF($B9="","",IF(ISNUMBER($F9),MAX(1,MIN(5,ROUND(6-$F9,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L9" s="41" t="str">
+        <f aca="false">IF($B9="","",IF(ISNUMBER($G9),MAX(1,MIN(5,ROUND(6-$G9,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M9" s="41" t="str">
+        <f aca="false">IF($B9="","",IF(AND(ISNUMBER($P9),ISNUMBER($O9)),MAX(1,MIN(5,ROUND(6-AVERAGE($P9,$O9),0))),IF(ISNUMBER($P9),MAX(1,MIN(5,ROUND(6-$P9,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O9" s="33" t="str">
+        <f aca="false">IF($B9="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B9),""))</f>
+        <v/>
+      </c>
+      <c r="P9" s="33" t="str">
+        <f aca="false">IF($B9="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B9),""))</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="37" t="str">
-        <f aca="false">IF(Suppliers!A8="","",Suppliers!A8)</f>
-        <v/>
-      </c>
-      <c r="B10" s="38" t="str">
-        <f aca="false">IF($A10="","",COUNTIF('Score Log'!$C$4:$C$203,$A10))</f>
-        <v/>
-      </c>
-      <c r="C10" s="39" t="str">
-        <f aca="false">IF($A10="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A10),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D10" s="39" t="str">
-        <f aca="false">IF($A10="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A10),1),"-"))</f>
+      <c r="A10" s="37"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="38" t="str">
+        <f aca="false">IF($B10="","",IF($C10="",COUNTIF('Score Log'!$C$4:$C$203,$B10),COUNTIFS('Score Log'!$C$4:$C$203,$B10,'Score Log'!$D$4:$D$203,$C10)))</f>
         <v/>
       </c>
       <c r="E10" s="39" t="str">
-        <f aca="false">IF($A10="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A10),1),"-"))</f>
+        <f aca="false">IF($B10="","",IFERROR(ROUND(IF($C10="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B10),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B10,'Score Log'!$D$4:$D$203,$C10)),1),"-"))</f>
         <v/>
       </c>
       <c r="F10" s="39" t="str">
-        <f aca="false">IF($A10="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A10),1),"-"))</f>
+        <f aca="false">IF($B10="","",IFERROR(ROUND(IF($C10="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B10),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B10,'Score Log'!$D$4:$D$203,$C10)),1),"-"))</f>
         <v/>
       </c>
       <c r="G10" s="39" t="str">
-        <f aca="false">IF($A10="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A10),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H10" s="40" t="str">
-        <f aca="false">IF($A10="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A10,'Score Log'!$U$4:$U$203,"Yes")/$B10,"-"))</f>
-        <v/>
-      </c>
-      <c r="I10" s="41" t="str">
-        <f aca="false">IF($A10="","",IF(ISNUMBER($D10),MAX(1,MIN(5,ROUND(6-$D10,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J10" s="41" t="str">
-        <f aca="false">IF($A10="","",IF(ISNUMBER($E10),MAX(1,MIN(5,ROUND(6-$E10,0))),"-"))</f>
+        <f aca="false">IF($B10="","",IFERROR(ROUND(IF($C10="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B10),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B10,'Score Log'!$D$4:$D$203,$C10)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H10" s="39" t="str">
+        <f aca="false">IF($B10="","",IFERROR(ROUND(IF($C10="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B10),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B10,'Score Log'!$D$4:$D$203,$C10)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I10" s="39" t="str">
+        <f aca="false">IF($B10="","",IFERROR(ROUND(IF($C10="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B10),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B10,'Score Log'!$D$4:$D$203,$C10)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J10" s="40" t="str">
+        <f aca="false">IF(OR($B10="",$D10=0),"",IFERROR(IF($C10="",COUNTIFS('Score Log'!$C$4:$C$203,$B10,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B10,'Score Log'!$D$4:$D$203,$C10,'Score Log'!$U$4:$U$203,"Yes"))/$D10,"-"))</f>
         <v/>
       </c>
       <c r="K10" s="41" t="str">
-        <f aca="false">IF($A10="","",IF(AND(ISNUMBER($F10),ISNUMBER($C10)),MAX(1,MIN(5,ROUND(6-AVERAGE($F10,$C10),0))),IF(ISNUMBER($F10),MAX(1,MIN(5,ROUND(6-$F10,0))),"-")))</f>
+        <f aca="false">IF($B10="","",IF(ISNUMBER($F10),MAX(1,MIN(5,ROUND(6-$F10,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L10" s="41" t="str">
+        <f aca="false">IF($B10="","",IF(ISNUMBER($G10),MAX(1,MIN(5,ROUND(6-$G10,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M10" s="41" t="str">
+        <f aca="false">IF($B10="","",IF(AND(ISNUMBER($P10),ISNUMBER($O10)),MAX(1,MIN(5,ROUND(6-AVERAGE($P10,$O10),0))),IF(ISNUMBER($P10),MAX(1,MIN(5,ROUND(6-$P10,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O10" s="33" t="str">
+        <f aca="false">IF($B10="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B10),""))</f>
+        <v/>
+      </c>
+      <c r="P10" s="33" t="str">
+        <f aca="false">IF($B10="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B10),""))</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="37" t="str">
-        <f aca="false">IF(Suppliers!A9="","",Suppliers!A9)</f>
-        <v/>
-      </c>
-      <c r="B11" s="38" t="str">
-        <f aca="false">IF($A11="","",COUNTIF('Score Log'!$C$4:$C$203,$A11))</f>
-        <v/>
-      </c>
-      <c r="C11" s="39" t="str">
-        <f aca="false">IF($A11="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A11),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D11" s="39" t="str">
-        <f aca="false">IF($A11="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A11),1),"-"))</f>
+      <c r="A11" s="37"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="38" t="str">
+        <f aca="false">IF($B11="","",IF($C11="",COUNTIF('Score Log'!$C$4:$C$203,$B11),COUNTIFS('Score Log'!$C$4:$C$203,$B11,'Score Log'!$D$4:$D$203,$C11)))</f>
         <v/>
       </c>
       <c r="E11" s="39" t="str">
-        <f aca="false">IF($A11="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A11),1),"-"))</f>
+        <f aca="false">IF($B11="","",IFERROR(ROUND(IF($C11="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B11),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B11,'Score Log'!$D$4:$D$203,$C11)),1),"-"))</f>
         <v/>
       </c>
       <c r="F11" s="39" t="str">
-        <f aca="false">IF($A11="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A11),1),"-"))</f>
+        <f aca="false">IF($B11="","",IFERROR(ROUND(IF($C11="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B11),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B11,'Score Log'!$D$4:$D$203,$C11)),1),"-"))</f>
         <v/>
       </c>
       <c r="G11" s="39" t="str">
-        <f aca="false">IF($A11="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A11),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H11" s="40" t="str">
-        <f aca="false">IF($A11="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A11,'Score Log'!$U$4:$U$203,"Yes")/$B11,"-"))</f>
-        <v/>
-      </c>
-      <c r="I11" s="41" t="str">
-        <f aca="false">IF($A11="","",IF(ISNUMBER($D11),MAX(1,MIN(5,ROUND(6-$D11,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J11" s="41" t="str">
-        <f aca="false">IF($A11="","",IF(ISNUMBER($E11),MAX(1,MIN(5,ROUND(6-$E11,0))),"-"))</f>
+        <f aca="false">IF($B11="","",IFERROR(ROUND(IF($C11="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B11),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B11,'Score Log'!$D$4:$D$203,$C11)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H11" s="39" t="str">
+        <f aca="false">IF($B11="","",IFERROR(ROUND(IF($C11="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B11),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B11,'Score Log'!$D$4:$D$203,$C11)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I11" s="39" t="str">
+        <f aca="false">IF($B11="","",IFERROR(ROUND(IF($C11="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B11),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B11,'Score Log'!$D$4:$D$203,$C11)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J11" s="40" t="str">
+        <f aca="false">IF(OR($B11="",$D11=0),"",IFERROR(IF($C11="",COUNTIFS('Score Log'!$C$4:$C$203,$B11,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B11,'Score Log'!$D$4:$D$203,$C11,'Score Log'!$U$4:$U$203,"Yes"))/$D11,"-"))</f>
         <v/>
       </c>
       <c r="K11" s="41" t="str">
-        <f aca="false">IF($A11="","",IF(AND(ISNUMBER($F11),ISNUMBER($C11)),MAX(1,MIN(5,ROUND(6-AVERAGE($F11,$C11),0))),IF(ISNUMBER($F11),MAX(1,MIN(5,ROUND(6-$F11,0))),"-")))</f>
+        <f aca="false">IF($B11="","",IF(ISNUMBER($F11),MAX(1,MIN(5,ROUND(6-$F11,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L11" s="41" t="str">
+        <f aca="false">IF($B11="","",IF(ISNUMBER($G11),MAX(1,MIN(5,ROUND(6-$G11,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M11" s="41" t="str">
+        <f aca="false">IF($B11="","",IF(AND(ISNUMBER($P11),ISNUMBER($O11)),MAX(1,MIN(5,ROUND(6-AVERAGE($P11,$O11),0))),IF(ISNUMBER($P11),MAX(1,MIN(5,ROUND(6-$P11,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O11" s="33" t="str">
+        <f aca="false">IF($B11="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B11),""))</f>
+        <v/>
+      </c>
+      <c r="P11" s="33" t="str">
+        <f aca="false">IF($B11="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B11),""))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37" t="str">
-        <f aca="false">IF(Suppliers!A10="","",Suppliers!A10)</f>
-        <v/>
-      </c>
-      <c r="B12" s="38" t="str">
-        <f aca="false">IF($A12="","",COUNTIF('Score Log'!$C$4:$C$203,$A12))</f>
-        <v/>
-      </c>
-      <c r="C12" s="39" t="str">
-        <f aca="false">IF($A12="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A12),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D12" s="39" t="str">
-        <f aca="false">IF($A12="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A12),1),"-"))</f>
+      <c r="A12" s="37"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="38" t="str">
+        <f aca="false">IF($B12="","",IF($C12="",COUNTIF('Score Log'!$C$4:$C$203,$B12),COUNTIFS('Score Log'!$C$4:$C$203,$B12,'Score Log'!$D$4:$D$203,$C12)))</f>
         <v/>
       </c>
       <c r="E12" s="39" t="str">
-        <f aca="false">IF($A12="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A12),1),"-"))</f>
+        <f aca="false">IF($B12="","",IFERROR(ROUND(IF($C12="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B12),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B12,'Score Log'!$D$4:$D$203,$C12)),1),"-"))</f>
         <v/>
       </c>
       <c r="F12" s="39" t="str">
-        <f aca="false">IF($A12="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A12),1),"-"))</f>
+        <f aca="false">IF($B12="","",IFERROR(ROUND(IF($C12="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B12),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B12,'Score Log'!$D$4:$D$203,$C12)),1),"-"))</f>
         <v/>
       </c>
       <c r="G12" s="39" t="str">
-        <f aca="false">IF($A12="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A12),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H12" s="40" t="str">
-        <f aca="false">IF($A12="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A12,'Score Log'!$U$4:$U$203,"Yes")/$B12,"-"))</f>
-        <v/>
-      </c>
-      <c r="I12" s="41" t="str">
-        <f aca="false">IF($A12="","",IF(ISNUMBER($D12),MAX(1,MIN(5,ROUND(6-$D12,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J12" s="41" t="str">
-        <f aca="false">IF($A12="","",IF(ISNUMBER($E12),MAX(1,MIN(5,ROUND(6-$E12,0))),"-"))</f>
+        <f aca="false">IF($B12="","",IFERROR(ROUND(IF($C12="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B12),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B12,'Score Log'!$D$4:$D$203,$C12)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H12" s="39" t="str">
+        <f aca="false">IF($B12="","",IFERROR(ROUND(IF($C12="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B12),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B12,'Score Log'!$D$4:$D$203,$C12)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I12" s="39" t="str">
+        <f aca="false">IF($B12="","",IFERROR(ROUND(IF($C12="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B12),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B12,'Score Log'!$D$4:$D$203,$C12)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J12" s="40" t="str">
+        <f aca="false">IF(OR($B12="",$D12=0),"",IFERROR(IF($C12="",COUNTIFS('Score Log'!$C$4:$C$203,$B12,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B12,'Score Log'!$D$4:$D$203,$C12,'Score Log'!$U$4:$U$203,"Yes"))/$D12,"-"))</f>
         <v/>
       </c>
       <c r="K12" s="41" t="str">
-        <f aca="false">IF($A12="","",IF(AND(ISNUMBER($F12),ISNUMBER($C12)),MAX(1,MIN(5,ROUND(6-AVERAGE($F12,$C12),0))),IF(ISNUMBER($F12),MAX(1,MIN(5,ROUND(6-$F12,0))),"-")))</f>
+        <f aca="false">IF($B12="","",IF(ISNUMBER($F12),MAX(1,MIN(5,ROUND(6-$F12,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L12" s="41" t="str">
+        <f aca="false">IF($B12="","",IF(ISNUMBER($G12),MAX(1,MIN(5,ROUND(6-$G12,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M12" s="41" t="str">
+        <f aca="false">IF($B12="","",IF(AND(ISNUMBER($P12),ISNUMBER($O12)),MAX(1,MIN(5,ROUND(6-AVERAGE($P12,$O12),0))),IF(ISNUMBER($P12),MAX(1,MIN(5,ROUND(6-$P12,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O12" s="33" t="str">
+        <f aca="false">IF($B12="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B12),""))</f>
+        <v/>
+      </c>
+      <c r="P12" s="33" t="str">
+        <f aca="false">IF($B12="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B12),""))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="37" t="str">
-        <f aca="false">IF(Suppliers!A11="","",Suppliers!A11)</f>
-        <v/>
-      </c>
-      <c r="B13" s="38" t="str">
-        <f aca="false">IF($A13="","",COUNTIF('Score Log'!$C$4:$C$203,$A13))</f>
-        <v/>
-      </c>
-      <c r="C13" s="39" t="str">
-        <f aca="false">IF($A13="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A13),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D13" s="39" t="str">
-        <f aca="false">IF($A13="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A13),1),"-"))</f>
+      <c r="A13" s="37"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="38" t="str">
+        <f aca="false">IF($B13="","",IF($C13="",COUNTIF('Score Log'!$C$4:$C$203,$B13),COUNTIFS('Score Log'!$C$4:$C$203,$B13,'Score Log'!$D$4:$D$203,$C13)))</f>
         <v/>
       </c>
       <c r="E13" s="39" t="str">
-        <f aca="false">IF($A13="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A13),1),"-"))</f>
+        <f aca="false">IF($B13="","",IFERROR(ROUND(IF($C13="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B13),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B13,'Score Log'!$D$4:$D$203,$C13)),1),"-"))</f>
         <v/>
       </c>
       <c r="F13" s="39" t="str">
-        <f aca="false">IF($A13="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A13),1),"-"))</f>
+        <f aca="false">IF($B13="","",IFERROR(ROUND(IF($C13="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B13),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B13,'Score Log'!$D$4:$D$203,$C13)),1),"-"))</f>
         <v/>
       </c>
       <c r="G13" s="39" t="str">
-        <f aca="false">IF($A13="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A13),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H13" s="40" t="str">
-        <f aca="false">IF($A13="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A13,'Score Log'!$U$4:$U$203,"Yes")/$B13,"-"))</f>
-        <v/>
-      </c>
-      <c r="I13" s="41" t="str">
-        <f aca="false">IF($A13="","",IF(ISNUMBER($D13),MAX(1,MIN(5,ROUND(6-$D13,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J13" s="41" t="str">
-        <f aca="false">IF($A13="","",IF(ISNUMBER($E13),MAX(1,MIN(5,ROUND(6-$E13,0))),"-"))</f>
+        <f aca="false">IF($B13="","",IFERROR(ROUND(IF($C13="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B13),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B13,'Score Log'!$D$4:$D$203,$C13)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H13" s="39" t="str">
+        <f aca="false">IF($B13="","",IFERROR(ROUND(IF($C13="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B13),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B13,'Score Log'!$D$4:$D$203,$C13)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I13" s="39" t="str">
+        <f aca="false">IF($B13="","",IFERROR(ROUND(IF($C13="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B13),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B13,'Score Log'!$D$4:$D$203,$C13)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J13" s="40" t="str">
+        <f aca="false">IF(OR($B13="",$D13=0),"",IFERROR(IF($C13="",COUNTIFS('Score Log'!$C$4:$C$203,$B13,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B13,'Score Log'!$D$4:$D$203,$C13,'Score Log'!$U$4:$U$203,"Yes"))/$D13,"-"))</f>
         <v/>
       </c>
       <c r="K13" s="41" t="str">
-        <f aca="false">IF($A13="","",IF(AND(ISNUMBER($F13),ISNUMBER($C13)),MAX(1,MIN(5,ROUND(6-AVERAGE($F13,$C13),0))),IF(ISNUMBER($F13),MAX(1,MIN(5,ROUND(6-$F13,0))),"-")))</f>
+        <f aca="false">IF($B13="","",IF(ISNUMBER($F13),MAX(1,MIN(5,ROUND(6-$F13,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L13" s="41" t="str">
+        <f aca="false">IF($B13="","",IF(ISNUMBER($G13),MAX(1,MIN(5,ROUND(6-$G13,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M13" s="41" t="str">
+        <f aca="false">IF($B13="","",IF(AND(ISNUMBER($P13),ISNUMBER($O13)),MAX(1,MIN(5,ROUND(6-AVERAGE($P13,$O13),0))),IF(ISNUMBER($P13),MAX(1,MIN(5,ROUND(6-$P13,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O13" s="33" t="str">
+        <f aca="false">IF($B13="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B13),""))</f>
+        <v/>
+      </c>
+      <c r="P13" s="33" t="str">
+        <f aca="false">IF($B13="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B13),""))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="37" t="str">
-        <f aca="false">IF(Suppliers!A12="","",Suppliers!A12)</f>
-        <v/>
-      </c>
-      <c r="B14" s="38" t="str">
-        <f aca="false">IF($A14="","",COUNTIF('Score Log'!$C$4:$C$203,$A14))</f>
-        <v/>
-      </c>
-      <c r="C14" s="39" t="str">
-        <f aca="false">IF($A14="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A14),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D14" s="39" t="str">
-        <f aca="false">IF($A14="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A14),1),"-"))</f>
+      <c r="A14" s="37"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="38" t="str">
+        <f aca="false">IF($B14="","",IF($C14="",COUNTIF('Score Log'!$C$4:$C$203,$B14),COUNTIFS('Score Log'!$C$4:$C$203,$B14,'Score Log'!$D$4:$D$203,$C14)))</f>
         <v/>
       </c>
       <c r="E14" s="39" t="str">
-        <f aca="false">IF($A14="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A14),1),"-"))</f>
+        <f aca="false">IF($B14="","",IFERROR(ROUND(IF($C14="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B14),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B14,'Score Log'!$D$4:$D$203,$C14)),1),"-"))</f>
         <v/>
       </c>
       <c r="F14" s="39" t="str">
-        <f aca="false">IF($A14="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A14),1),"-"))</f>
+        <f aca="false">IF($B14="","",IFERROR(ROUND(IF($C14="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B14),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B14,'Score Log'!$D$4:$D$203,$C14)),1),"-"))</f>
         <v/>
       </c>
       <c r="G14" s="39" t="str">
-        <f aca="false">IF($A14="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A14),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H14" s="40" t="str">
-        <f aca="false">IF($A14="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A14,'Score Log'!$U$4:$U$203,"Yes")/$B14,"-"))</f>
-        <v/>
-      </c>
-      <c r="I14" s="41" t="str">
-        <f aca="false">IF($A14="","",IF(ISNUMBER($D14),MAX(1,MIN(5,ROUND(6-$D14,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J14" s="41" t="str">
-        <f aca="false">IF($A14="","",IF(ISNUMBER($E14),MAX(1,MIN(5,ROUND(6-$E14,0))),"-"))</f>
+        <f aca="false">IF($B14="","",IFERROR(ROUND(IF($C14="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B14),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B14,'Score Log'!$D$4:$D$203,$C14)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H14" s="39" t="str">
+        <f aca="false">IF($B14="","",IFERROR(ROUND(IF($C14="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B14),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B14,'Score Log'!$D$4:$D$203,$C14)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I14" s="39" t="str">
+        <f aca="false">IF($B14="","",IFERROR(ROUND(IF($C14="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B14),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B14,'Score Log'!$D$4:$D$203,$C14)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J14" s="40" t="str">
+        <f aca="false">IF(OR($B14="",$D14=0),"",IFERROR(IF($C14="",COUNTIFS('Score Log'!$C$4:$C$203,$B14,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B14,'Score Log'!$D$4:$D$203,$C14,'Score Log'!$U$4:$U$203,"Yes"))/$D14,"-"))</f>
         <v/>
       </c>
       <c r="K14" s="41" t="str">
-        <f aca="false">IF($A14="","",IF(AND(ISNUMBER($F14),ISNUMBER($C14)),MAX(1,MIN(5,ROUND(6-AVERAGE($F14,$C14),0))),IF(ISNUMBER($F14),MAX(1,MIN(5,ROUND(6-$F14,0))),"-")))</f>
+        <f aca="false">IF($B14="","",IF(ISNUMBER($F14),MAX(1,MIN(5,ROUND(6-$F14,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L14" s="41" t="str">
+        <f aca="false">IF($B14="","",IF(ISNUMBER($G14),MAX(1,MIN(5,ROUND(6-$G14,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M14" s="41" t="str">
+        <f aca="false">IF($B14="","",IF(AND(ISNUMBER($P14),ISNUMBER($O14)),MAX(1,MIN(5,ROUND(6-AVERAGE($P14,$O14),0))),IF(ISNUMBER($P14),MAX(1,MIN(5,ROUND(6-$P14,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O14" s="33" t="str">
+        <f aca="false">IF($B14="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B14),""))</f>
+        <v/>
+      </c>
+      <c r="P14" s="33" t="str">
+        <f aca="false">IF($B14="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B14),""))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="37" t="str">
-        <f aca="false">IF(Suppliers!A13="","",Suppliers!A13)</f>
-        <v/>
-      </c>
-      <c r="B15" s="38" t="str">
-        <f aca="false">IF($A15="","",COUNTIF('Score Log'!$C$4:$C$203,$A15))</f>
-        <v/>
-      </c>
-      <c r="C15" s="39" t="str">
-        <f aca="false">IF($A15="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A15),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D15" s="39" t="str">
-        <f aca="false">IF($A15="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A15),1),"-"))</f>
+      <c r="A15" s="37"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="38" t="str">
+        <f aca="false">IF($B15="","",IF($C15="",COUNTIF('Score Log'!$C$4:$C$203,$B15),COUNTIFS('Score Log'!$C$4:$C$203,$B15,'Score Log'!$D$4:$D$203,$C15)))</f>
         <v/>
       </c>
       <c r="E15" s="39" t="str">
-        <f aca="false">IF($A15="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A15),1),"-"))</f>
+        <f aca="false">IF($B15="","",IFERROR(ROUND(IF($C15="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B15),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B15,'Score Log'!$D$4:$D$203,$C15)),1),"-"))</f>
         <v/>
       </c>
       <c r="F15" s="39" t="str">
-        <f aca="false">IF($A15="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A15),1),"-"))</f>
+        <f aca="false">IF($B15="","",IFERROR(ROUND(IF($C15="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B15),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B15,'Score Log'!$D$4:$D$203,$C15)),1),"-"))</f>
         <v/>
       </c>
       <c r="G15" s="39" t="str">
-        <f aca="false">IF($A15="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A15),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H15" s="40" t="str">
-        <f aca="false">IF($A15="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A15,'Score Log'!$U$4:$U$203,"Yes")/$B15,"-"))</f>
-        <v/>
-      </c>
-      <c r="I15" s="41" t="str">
-        <f aca="false">IF($A15="","",IF(ISNUMBER($D15),MAX(1,MIN(5,ROUND(6-$D15,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J15" s="41" t="str">
-        <f aca="false">IF($A15="","",IF(ISNUMBER($E15),MAX(1,MIN(5,ROUND(6-$E15,0))),"-"))</f>
+        <f aca="false">IF($B15="","",IFERROR(ROUND(IF($C15="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B15),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B15,'Score Log'!$D$4:$D$203,$C15)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H15" s="39" t="str">
+        <f aca="false">IF($B15="","",IFERROR(ROUND(IF($C15="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B15),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B15,'Score Log'!$D$4:$D$203,$C15)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I15" s="39" t="str">
+        <f aca="false">IF($B15="","",IFERROR(ROUND(IF($C15="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B15),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B15,'Score Log'!$D$4:$D$203,$C15)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J15" s="40" t="str">
+        <f aca="false">IF(OR($B15="",$D15=0),"",IFERROR(IF($C15="",COUNTIFS('Score Log'!$C$4:$C$203,$B15,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B15,'Score Log'!$D$4:$D$203,$C15,'Score Log'!$U$4:$U$203,"Yes"))/$D15,"-"))</f>
         <v/>
       </c>
       <c r="K15" s="41" t="str">
-        <f aca="false">IF($A15="","",IF(AND(ISNUMBER($F15),ISNUMBER($C15)),MAX(1,MIN(5,ROUND(6-AVERAGE($F15,$C15),0))),IF(ISNUMBER($F15),MAX(1,MIN(5,ROUND(6-$F15,0))),"-")))</f>
+        <f aca="false">IF($B15="","",IF(ISNUMBER($F15),MAX(1,MIN(5,ROUND(6-$F15,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L15" s="41" t="str">
+        <f aca="false">IF($B15="","",IF(ISNUMBER($G15),MAX(1,MIN(5,ROUND(6-$G15,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M15" s="41" t="str">
+        <f aca="false">IF($B15="","",IF(AND(ISNUMBER($P15),ISNUMBER($O15)),MAX(1,MIN(5,ROUND(6-AVERAGE($P15,$O15),0))),IF(ISNUMBER($P15),MAX(1,MIN(5,ROUND(6-$P15,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O15" s="33" t="str">
+        <f aca="false">IF($B15="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B15),""))</f>
+        <v/>
+      </c>
+      <c r="P15" s="33" t="str">
+        <f aca="false">IF($B15="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B15),""))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="37" t="str">
-        <f aca="false">IF(Suppliers!A14="","",Suppliers!A14)</f>
-        <v/>
-      </c>
-      <c r="B16" s="38" t="str">
-        <f aca="false">IF($A16="","",COUNTIF('Score Log'!$C$4:$C$203,$A16))</f>
-        <v/>
-      </c>
-      <c r="C16" s="39" t="str">
-        <f aca="false">IF($A16="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A16),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D16" s="39" t="str">
-        <f aca="false">IF($A16="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A16),1),"-"))</f>
+      <c r="A16" s="37"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="38" t="str">
+        <f aca="false">IF($B16="","",IF($C16="",COUNTIF('Score Log'!$C$4:$C$203,$B16),COUNTIFS('Score Log'!$C$4:$C$203,$B16,'Score Log'!$D$4:$D$203,$C16)))</f>
         <v/>
       </c>
       <c r="E16" s="39" t="str">
-        <f aca="false">IF($A16="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A16),1),"-"))</f>
+        <f aca="false">IF($B16="","",IFERROR(ROUND(IF($C16="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B16),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B16,'Score Log'!$D$4:$D$203,$C16)),1),"-"))</f>
         <v/>
       </c>
       <c r="F16" s="39" t="str">
-        <f aca="false">IF($A16="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A16),1),"-"))</f>
+        <f aca="false">IF($B16="","",IFERROR(ROUND(IF($C16="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B16),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B16,'Score Log'!$D$4:$D$203,$C16)),1),"-"))</f>
         <v/>
       </c>
       <c r="G16" s="39" t="str">
-        <f aca="false">IF($A16="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A16),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H16" s="40" t="str">
-        <f aca="false">IF($A16="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A16,'Score Log'!$U$4:$U$203,"Yes")/$B16,"-"))</f>
-        <v/>
-      </c>
-      <c r="I16" s="41" t="str">
-        <f aca="false">IF($A16="","",IF(ISNUMBER($D16),MAX(1,MIN(5,ROUND(6-$D16,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J16" s="41" t="str">
-        <f aca="false">IF($A16="","",IF(ISNUMBER($E16),MAX(1,MIN(5,ROUND(6-$E16,0))),"-"))</f>
+        <f aca="false">IF($B16="","",IFERROR(ROUND(IF($C16="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B16),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B16,'Score Log'!$D$4:$D$203,$C16)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H16" s="39" t="str">
+        <f aca="false">IF($B16="","",IFERROR(ROUND(IF($C16="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B16),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B16,'Score Log'!$D$4:$D$203,$C16)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I16" s="39" t="str">
+        <f aca="false">IF($B16="","",IFERROR(ROUND(IF($C16="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B16),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B16,'Score Log'!$D$4:$D$203,$C16)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J16" s="40" t="str">
+        <f aca="false">IF(OR($B16="",$D16=0),"",IFERROR(IF($C16="",COUNTIFS('Score Log'!$C$4:$C$203,$B16,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B16,'Score Log'!$D$4:$D$203,$C16,'Score Log'!$U$4:$U$203,"Yes"))/$D16,"-"))</f>
         <v/>
       </c>
       <c r="K16" s="41" t="str">
-        <f aca="false">IF($A16="","",IF(AND(ISNUMBER($F16),ISNUMBER($C16)),MAX(1,MIN(5,ROUND(6-AVERAGE($F16,$C16),0))),IF(ISNUMBER($F16),MAX(1,MIN(5,ROUND(6-$F16,0))),"-")))</f>
+        <f aca="false">IF($B16="","",IF(ISNUMBER($F16),MAX(1,MIN(5,ROUND(6-$F16,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L16" s="41" t="str">
+        <f aca="false">IF($B16="","",IF(ISNUMBER($G16),MAX(1,MIN(5,ROUND(6-$G16,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M16" s="41" t="str">
+        <f aca="false">IF($B16="","",IF(AND(ISNUMBER($P16),ISNUMBER($O16)),MAX(1,MIN(5,ROUND(6-AVERAGE($P16,$O16),0))),IF(ISNUMBER($P16),MAX(1,MIN(5,ROUND(6-$P16,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O16" s="33" t="str">
+        <f aca="false">IF($B16="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B16),""))</f>
+        <v/>
+      </c>
+      <c r="P16" s="33" t="str">
+        <f aca="false">IF($B16="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B16),""))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="37" t="str">
-        <f aca="false">IF(Suppliers!A15="","",Suppliers!A15)</f>
-        <v/>
-      </c>
-      <c r="B17" s="38" t="str">
-        <f aca="false">IF($A17="","",COUNTIF('Score Log'!$C$4:$C$203,$A17))</f>
-        <v/>
-      </c>
-      <c r="C17" s="39" t="str">
-        <f aca="false">IF($A17="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A17),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D17" s="39" t="str">
-        <f aca="false">IF($A17="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A17),1),"-"))</f>
+      <c r="A17" s="37"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="38" t="str">
+        <f aca="false">IF($B17="","",IF($C17="",COUNTIF('Score Log'!$C$4:$C$203,$B17),COUNTIFS('Score Log'!$C$4:$C$203,$B17,'Score Log'!$D$4:$D$203,$C17)))</f>
         <v/>
       </c>
       <c r="E17" s="39" t="str">
-        <f aca="false">IF($A17="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A17),1),"-"))</f>
+        <f aca="false">IF($B17="","",IFERROR(ROUND(IF($C17="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B17),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B17,'Score Log'!$D$4:$D$203,$C17)),1),"-"))</f>
         <v/>
       </c>
       <c r="F17" s="39" t="str">
-        <f aca="false">IF($A17="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A17),1),"-"))</f>
+        <f aca="false">IF($B17="","",IFERROR(ROUND(IF($C17="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B17),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B17,'Score Log'!$D$4:$D$203,$C17)),1),"-"))</f>
         <v/>
       </c>
       <c r="G17" s="39" t="str">
-        <f aca="false">IF($A17="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A17),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H17" s="40" t="str">
-        <f aca="false">IF($A17="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A17,'Score Log'!$U$4:$U$203,"Yes")/$B17,"-"))</f>
-        <v/>
-      </c>
-      <c r="I17" s="41" t="str">
-        <f aca="false">IF($A17="","",IF(ISNUMBER($D17),MAX(1,MIN(5,ROUND(6-$D17,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J17" s="41" t="str">
-        <f aca="false">IF($A17="","",IF(ISNUMBER($E17),MAX(1,MIN(5,ROUND(6-$E17,0))),"-"))</f>
+        <f aca="false">IF($B17="","",IFERROR(ROUND(IF($C17="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B17),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B17,'Score Log'!$D$4:$D$203,$C17)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H17" s="39" t="str">
+        <f aca="false">IF($B17="","",IFERROR(ROUND(IF($C17="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B17),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B17,'Score Log'!$D$4:$D$203,$C17)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I17" s="39" t="str">
+        <f aca="false">IF($B17="","",IFERROR(ROUND(IF($C17="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B17),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B17,'Score Log'!$D$4:$D$203,$C17)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J17" s="40" t="str">
+        <f aca="false">IF(OR($B17="",$D17=0),"",IFERROR(IF($C17="",COUNTIFS('Score Log'!$C$4:$C$203,$B17,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B17,'Score Log'!$D$4:$D$203,$C17,'Score Log'!$U$4:$U$203,"Yes"))/$D17,"-"))</f>
         <v/>
       </c>
       <c r="K17" s="41" t="str">
-        <f aca="false">IF($A17="","",IF(AND(ISNUMBER($F17),ISNUMBER($C17)),MAX(1,MIN(5,ROUND(6-AVERAGE($F17,$C17),0))),IF(ISNUMBER($F17),MAX(1,MIN(5,ROUND(6-$F17,0))),"-")))</f>
+        <f aca="false">IF($B17="","",IF(ISNUMBER($F17),MAX(1,MIN(5,ROUND(6-$F17,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L17" s="41" t="str">
+        <f aca="false">IF($B17="","",IF(ISNUMBER($G17),MAX(1,MIN(5,ROUND(6-$G17,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M17" s="41" t="str">
+        <f aca="false">IF($B17="","",IF(AND(ISNUMBER($P17),ISNUMBER($O17)),MAX(1,MIN(5,ROUND(6-AVERAGE($P17,$O17),0))),IF(ISNUMBER($P17),MAX(1,MIN(5,ROUND(6-$P17,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O17" s="33" t="str">
+        <f aca="false">IF($B17="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B17),""))</f>
+        <v/>
+      </c>
+      <c r="P17" s="33" t="str">
+        <f aca="false">IF($B17="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B17),""))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="37" t="str">
-        <f aca="false">IF(Suppliers!A16="","",Suppliers!A16)</f>
-        <v/>
-      </c>
-      <c r="B18" s="38" t="str">
-        <f aca="false">IF($A18="","",COUNTIF('Score Log'!$C$4:$C$203,$A18))</f>
-        <v/>
-      </c>
-      <c r="C18" s="39" t="str">
-        <f aca="false">IF($A18="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A18),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D18" s="39" t="str">
-        <f aca="false">IF($A18="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A18),1),"-"))</f>
+      <c r="A18" s="37"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="38" t="str">
+        <f aca="false">IF($B18="","",IF($C18="",COUNTIF('Score Log'!$C$4:$C$203,$B18),COUNTIFS('Score Log'!$C$4:$C$203,$B18,'Score Log'!$D$4:$D$203,$C18)))</f>
         <v/>
       </c>
       <c r="E18" s="39" t="str">
-        <f aca="false">IF($A18="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A18),1),"-"))</f>
+        <f aca="false">IF($B18="","",IFERROR(ROUND(IF($C18="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B18),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B18,'Score Log'!$D$4:$D$203,$C18)),1),"-"))</f>
         <v/>
       </c>
       <c r="F18" s="39" t="str">
-        <f aca="false">IF($A18="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A18),1),"-"))</f>
+        <f aca="false">IF($B18="","",IFERROR(ROUND(IF($C18="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B18),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B18,'Score Log'!$D$4:$D$203,$C18)),1),"-"))</f>
         <v/>
       </c>
       <c r="G18" s="39" t="str">
-        <f aca="false">IF($A18="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A18),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H18" s="40" t="str">
-        <f aca="false">IF($A18="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A18,'Score Log'!$U$4:$U$203,"Yes")/$B18,"-"))</f>
-        <v/>
-      </c>
-      <c r="I18" s="41" t="str">
-        <f aca="false">IF($A18="","",IF(ISNUMBER($D18),MAX(1,MIN(5,ROUND(6-$D18,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J18" s="41" t="str">
-        <f aca="false">IF($A18="","",IF(ISNUMBER($E18),MAX(1,MIN(5,ROUND(6-$E18,0))),"-"))</f>
+        <f aca="false">IF($B18="","",IFERROR(ROUND(IF($C18="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B18),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B18,'Score Log'!$D$4:$D$203,$C18)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H18" s="39" t="str">
+        <f aca="false">IF($B18="","",IFERROR(ROUND(IF($C18="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B18),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B18,'Score Log'!$D$4:$D$203,$C18)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I18" s="39" t="str">
+        <f aca="false">IF($B18="","",IFERROR(ROUND(IF($C18="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B18),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B18,'Score Log'!$D$4:$D$203,$C18)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J18" s="40" t="str">
+        <f aca="false">IF(OR($B18="",$D18=0),"",IFERROR(IF($C18="",COUNTIFS('Score Log'!$C$4:$C$203,$B18,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B18,'Score Log'!$D$4:$D$203,$C18,'Score Log'!$U$4:$U$203,"Yes"))/$D18,"-"))</f>
         <v/>
       </c>
       <c r="K18" s="41" t="str">
-        <f aca="false">IF($A18="","",IF(AND(ISNUMBER($F18),ISNUMBER($C18)),MAX(1,MIN(5,ROUND(6-AVERAGE($F18,$C18),0))),IF(ISNUMBER($F18),MAX(1,MIN(5,ROUND(6-$F18,0))),"-")))</f>
+        <f aca="false">IF($B18="","",IF(ISNUMBER($F18),MAX(1,MIN(5,ROUND(6-$F18,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L18" s="41" t="str">
+        <f aca="false">IF($B18="","",IF(ISNUMBER($G18),MAX(1,MIN(5,ROUND(6-$G18,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M18" s="41" t="str">
+        <f aca="false">IF($B18="","",IF(AND(ISNUMBER($P18),ISNUMBER($O18)),MAX(1,MIN(5,ROUND(6-AVERAGE($P18,$O18),0))),IF(ISNUMBER($P18),MAX(1,MIN(5,ROUND(6-$P18,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O18" s="33" t="str">
+        <f aca="false">IF($B18="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B18),""))</f>
+        <v/>
+      </c>
+      <c r="P18" s="33" t="str">
+        <f aca="false">IF($B18="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B18),""))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37" t="str">
-        <f aca="false">IF(Suppliers!A17="","",Suppliers!A17)</f>
-        <v/>
-      </c>
-      <c r="B19" s="38" t="str">
-        <f aca="false">IF($A19="","",COUNTIF('Score Log'!$C$4:$C$203,$A19))</f>
-        <v/>
-      </c>
-      <c r="C19" s="39" t="str">
-        <f aca="false">IF($A19="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A19),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D19" s="39" t="str">
-        <f aca="false">IF($A19="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A19),1),"-"))</f>
+      <c r="A19" s="37"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="38" t="str">
+        <f aca="false">IF($B19="","",IF($C19="",COUNTIF('Score Log'!$C$4:$C$203,$B19),COUNTIFS('Score Log'!$C$4:$C$203,$B19,'Score Log'!$D$4:$D$203,$C19)))</f>
         <v/>
       </c>
       <c r="E19" s="39" t="str">
-        <f aca="false">IF($A19="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A19),1),"-"))</f>
+        <f aca="false">IF($B19="","",IFERROR(ROUND(IF($C19="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B19),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B19,'Score Log'!$D$4:$D$203,$C19)),1),"-"))</f>
         <v/>
       </c>
       <c r="F19" s="39" t="str">
-        <f aca="false">IF($A19="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A19),1),"-"))</f>
+        <f aca="false">IF($B19="","",IFERROR(ROUND(IF($C19="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B19),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B19,'Score Log'!$D$4:$D$203,$C19)),1),"-"))</f>
         <v/>
       </c>
       <c r="G19" s="39" t="str">
-        <f aca="false">IF($A19="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A19),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H19" s="40" t="str">
-        <f aca="false">IF($A19="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A19,'Score Log'!$U$4:$U$203,"Yes")/$B19,"-"))</f>
-        <v/>
-      </c>
-      <c r="I19" s="41" t="str">
-        <f aca="false">IF($A19="","",IF(ISNUMBER($D19),MAX(1,MIN(5,ROUND(6-$D19,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J19" s="41" t="str">
-        <f aca="false">IF($A19="","",IF(ISNUMBER($E19),MAX(1,MIN(5,ROUND(6-$E19,0))),"-"))</f>
+        <f aca="false">IF($B19="","",IFERROR(ROUND(IF($C19="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B19),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B19,'Score Log'!$D$4:$D$203,$C19)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H19" s="39" t="str">
+        <f aca="false">IF($B19="","",IFERROR(ROUND(IF($C19="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B19),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B19,'Score Log'!$D$4:$D$203,$C19)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I19" s="39" t="str">
+        <f aca="false">IF($B19="","",IFERROR(ROUND(IF($C19="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B19),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B19,'Score Log'!$D$4:$D$203,$C19)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J19" s="40" t="str">
+        <f aca="false">IF(OR($B19="",$D19=0),"",IFERROR(IF($C19="",COUNTIFS('Score Log'!$C$4:$C$203,$B19,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B19,'Score Log'!$D$4:$D$203,$C19,'Score Log'!$U$4:$U$203,"Yes"))/$D19,"-"))</f>
         <v/>
       </c>
       <c r="K19" s="41" t="str">
-        <f aca="false">IF($A19="","",IF(AND(ISNUMBER($F19),ISNUMBER($C19)),MAX(1,MIN(5,ROUND(6-AVERAGE($F19,$C19),0))),IF(ISNUMBER($F19),MAX(1,MIN(5,ROUND(6-$F19,0))),"-")))</f>
+        <f aca="false">IF($B19="","",IF(ISNUMBER($F19),MAX(1,MIN(5,ROUND(6-$F19,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L19" s="41" t="str">
+        <f aca="false">IF($B19="","",IF(ISNUMBER($G19),MAX(1,MIN(5,ROUND(6-$G19,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M19" s="41" t="str">
+        <f aca="false">IF($B19="","",IF(AND(ISNUMBER($P19),ISNUMBER($O19)),MAX(1,MIN(5,ROUND(6-AVERAGE($P19,$O19),0))),IF(ISNUMBER($P19),MAX(1,MIN(5,ROUND(6-$P19,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O19" s="33" t="str">
+        <f aca="false">IF($B19="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B19),""))</f>
+        <v/>
+      </c>
+      <c r="P19" s="33" t="str">
+        <f aca="false">IF($B19="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B19),""))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="37" t="str">
-        <f aca="false">IF(Suppliers!A18="","",Suppliers!A18)</f>
-        <v/>
-      </c>
-      <c r="B20" s="38" t="str">
-        <f aca="false">IF($A20="","",COUNTIF('Score Log'!$C$4:$C$203,$A20))</f>
-        <v/>
-      </c>
-      <c r="C20" s="39" t="str">
-        <f aca="false">IF($A20="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A20),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D20" s="39" t="str">
-        <f aca="false">IF($A20="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A20),1),"-"))</f>
+      <c r="A20" s="37"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="38" t="str">
+        <f aca="false">IF($B20="","",IF($C20="",COUNTIF('Score Log'!$C$4:$C$203,$B20),COUNTIFS('Score Log'!$C$4:$C$203,$B20,'Score Log'!$D$4:$D$203,$C20)))</f>
         <v/>
       </c>
       <c r="E20" s="39" t="str">
-        <f aca="false">IF($A20="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A20),1),"-"))</f>
+        <f aca="false">IF($B20="","",IFERROR(ROUND(IF($C20="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B20),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B20,'Score Log'!$D$4:$D$203,$C20)),1),"-"))</f>
         <v/>
       </c>
       <c r="F20" s="39" t="str">
-        <f aca="false">IF($A20="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A20),1),"-"))</f>
+        <f aca="false">IF($B20="","",IFERROR(ROUND(IF($C20="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B20),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B20,'Score Log'!$D$4:$D$203,$C20)),1),"-"))</f>
         <v/>
       </c>
       <c r="G20" s="39" t="str">
-        <f aca="false">IF($A20="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A20),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H20" s="40" t="str">
-        <f aca="false">IF($A20="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A20,'Score Log'!$U$4:$U$203,"Yes")/$B20,"-"))</f>
-        <v/>
-      </c>
-      <c r="I20" s="41" t="str">
-        <f aca="false">IF($A20="","",IF(ISNUMBER($D20),MAX(1,MIN(5,ROUND(6-$D20,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J20" s="41" t="str">
-        <f aca="false">IF($A20="","",IF(ISNUMBER($E20),MAX(1,MIN(5,ROUND(6-$E20,0))),"-"))</f>
+        <f aca="false">IF($B20="","",IFERROR(ROUND(IF($C20="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B20),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B20,'Score Log'!$D$4:$D$203,$C20)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H20" s="39" t="str">
+        <f aca="false">IF($B20="","",IFERROR(ROUND(IF($C20="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B20),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B20,'Score Log'!$D$4:$D$203,$C20)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I20" s="39" t="str">
+        <f aca="false">IF($B20="","",IFERROR(ROUND(IF($C20="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B20),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B20,'Score Log'!$D$4:$D$203,$C20)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J20" s="40" t="str">
+        <f aca="false">IF(OR($B20="",$D20=0),"",IFERROR(IF($C20="",COUNTIFS('Score Log'!$C$4:$C$203,$B20,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B20,'Score Log'!$D$4:$D$203,$C20,'Score Log'!$U$4:$U$203,"Yes"))/$D20,"-"))</f>
         <v/>
       </c>
       <c r="K20" s="41" t="str">
-        <f aca="false">IF($A20="","",IF(AND(ISNUMBER($F20),ISNUMBER($C20)),MAX(1,MIN(5,ROUND(6-AVERAGE($F20,$C20),0))),IF(ISNUMBER($F20),MAX(1,MIN(5,ROUND(6-$F20,0))),"-")))</f>
+        <f aca="false">IF($B20="","",IF(ISNUMBER($F20),MAX(1,MIN(5,ROUND(6-$F20,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L20" s="41" t="str">
+        <f aca="false">IF($B20="","",IF(ISNUMBER($G20),MAX(1,MIN(5,ROUND(6-$G20,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M20" s="41" t="str">
+        <f aca="false">IF($B20="","",IF(AND(ISNUMBER($P20),ISNUMBER($O20)),MAX(1,MIN(5,ROUND(6-AVERAGE($P20,$O20),0))),IF(ISNUMBER($P20),MAX(1,MIN(5,ROUND(6-$P20,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O20" s="33" t="str">
+        <f aca="false">IF($B20="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B20),""))</f>
+        <v/>
+      </c>
+      <c r="P20" s="33" t="str">
+        <f aca="false">IF($B20="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B20),""))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="37" t="str">
-        <f aca="false">IF(Suppliers!A19="","",Suppliers!A19)</f>
-        <v/>
-      </c>
-      <c r="B21" s="38" t="str">
-        <f aca="false">IF($A21="","",COUNTIF('Score Log'!$C$4:$C$203,$A21))</f>
-        <v/>
-      </c>
-      <c r="C21" s="39" t="str">
-        <f aca="false">IF($A21="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A21),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D21" s="39" t="str">
-        <f aca="false">IF($A21="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A21),1),"-"))</f>
+      <c r="A21" s="37"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="38" t="str">
+        <f aca="false">IF($B21="","",IF($C21="",COUNTIF('Score Log'!$C$4:$C$203,$B21),COUNTIFS('Score Log'!$C$4:$C$203,$B21,'Score Log'!$D$4:$D$203,$C21)))</f>
         <v/>
       </c>
       <c r="E21" s="39" t="str">
-        <f aca="false">IF($A21="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A21),1),"-"))</f>
+        <f aca="false">IF($B21="","",IFERROR(ROUND(IF($C21="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B21),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B21,'Score Log'!$D$4:$D$203,$C21)),1),"-"))</f>
         <v/>
       </c>
       <c r="F21" s="39" t="str">
-        <f aca="false">IF($A21="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A21),1),"-"))</f>
+        <f aca="false">IF($B21="","",IFERROR(ROUND(IF($C21="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B21),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B21,'Score Log'!$D$4:$D$203,$C21)),1),"-"))</f>
         <v/>
       </c>
       <c r="G21" s="39" t="str">
-        <f aca="false">IF($A21="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A21),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H21" s="40" t="str">
-        <f aca="false">IF($A21="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A21,'Score Log'!$U$4:$U$203,"Yes")/$B21,"-"))</f>
-        <v/>
-      </c>
-      <c r="I21" s="41" t="str">
-        <f aca="false">IF($A21="","",IF(ISNUMBER($D21),MAX(1,MIN(5,ROUND(6-$D21,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J21" s="41" t="str">
-        <f aca="false">IF($A21="","",IF(ISNUMBER($E21),MAX(1,MIN(5,ROUND(6-$E21,0))),"-"))</f>
+        <f aca="false">IF($B21="","",IFERROR(ROUND(IF($C21="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B21),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B21,'Score Log'!$D$4:$D$203,$C21)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H21" s="39" t="str">
+        <f aca="false">IF($B21="","",IFERROR(ROUND(IF($C21="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B21),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B21,'Score Log'!$D$4:$D$203,$C21)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I21" s="39" t="str">
+        <f aca="false">IF($B21="","",IFERROR(ROUND(IF($C21="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B21),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B21,'Score Log'!$D$4:$D$203,$C21)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J21" s="40" t="str">
+        <f aca="false">IF(OR($B21="",$D21=0),"",IFERROR(IF($C21="",COUNTIFS('Score Log'!$C$4:$C$203,$B21,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B21,'Score Log'!$D$4:$D$203,$C21,'Score Log'!$U$4:$U$203,"Yes"))/$D21,"-"))</f>
         <v/>
       </c>
       <c r="K21" s="41" t="str">
-        <f aca="false">IF($A21="","",IF(AND(ISNUMBER($F21),ISNUMBER($C21)),MAX(1,MIN(5,ROUND(6-AVERAGE($F21,$C21),0))),IF(ISNUMBER($F21),MAX(1,MIN(5,ROUND(6-$F21,0))),"-")))</f>
+        <f aca="false">IF($B21="","",IF(ISNUMBER($F21),MAX(1,MIN(5,ROUND(6-$F21,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L21" s="41" t="str">
+        <f aca="false">IF($B21="","",IF(ISNUMBER($G21),MAX(1,MIN(5,ROUND(6-$G21,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M21" s="41" t="str">
+        <f aca="false">IF($B21="","",IF(AND(ISNUMBER($P21),ISNUMBER($O21)),MAX(1,MIN(5,ROUND(6-AVERAGE($P21,$O21),0))),IF(ISNUMBER($P21),MAX(1,MIN(5,ROUND(6-$P21,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O21" s="33" t="str">
+        <f aca="false">IF($B21="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B21),""))</f>
+        <v/>
+      </c>
+      <c r="P21" s="33" t="str">
+        <f aca="false">IF($B21="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B21),""))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="37" t="str">
-        <f aca="false">IF(Suppliers!A20="","",Suppliers!A20)</f>
-        <v/>
-      </c>
-      <c r="B22" s="38" t="str">
-        <f aca="false">IF($A22="","",COUNTIF('Score Log'!$C$4:$C$203,$A22))</f>
-        <v/>
-      </c>
-      <c r="C22" s="39" t="str">
-        <f aca="false">IF($A22="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A22),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D22" s="39" t="str">
-        <f aca="false">IF($A22="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A22),1),"-"))</f>
+      <c r="A22" s="37"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="38" t="str">
+        <f aca="false">IF($B22="","",IF($C22="",COUNTIF('Score Log'!$C$4:$C$203,$B22),COUNTIFS('Score Log'!$C$4:$C$203,$B22,'Score Log'!$D$4:$D$203,$C22)))</f>
         <v/>
       </c>
       <c r="E22" s="39" t="str">
-        <f aca="false">IF($A22="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A22),1),"-"))</f>
+        <f aca="false">IF($B22="","",IFERROR(ROUND(IF($C22="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B22),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B22,'Score Log'!$D$4:$D$203,$C22)),1),"-"))</f>
         <v/>
       </c>
       <c r="F22" s="39" t="str">
-        <f aca="false">IF($A22="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A22),1),"-"))</f>
+        <f aca="false">IF($B22="","",IFERROR(ROUND(IF($C22="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B22),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B22,'Score Log'!$D$4:$D$203,$C22)),1),"-"))</f>
         <v/>
       </c>
       <c r="G22" s="39" t="str">
-        <f aca="false">IF($A22="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A22),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H22" s="40" t="str">
-        <f aca="false">IF($A22="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A22,'Score Log'!$U$4:$U$203,"Yes")/$B22,"-"))</f>
-        <v/>
-      </c>
-      <c r="I22" s="41" t="str">
-        <f aca="false">IF($A22="","",IF(ISNUMBER($D22),MAX(1,MIN(5,ROUND(6-$D22,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J22" s="41" t="str">
-        <f aca="false">IF($A22="","",IF(ISNUMBER($E22),MAX(1,MIN(5,ROUND(6-$E22,0))),"-"))</f>
+        <f aca="false">IF($B22="","",IFERROR(ROUND(IF($C22="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B22),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B22,'Score Log'!$D$4:$D$203,$C22)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H22" s="39" t="str">
+        <f aca="false">IF($B22="","",IFERROR(ROUND(IF($C22="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B22),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B22,'Score Log'!$D$4:$D$203,$C22)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I22" s="39" t="str">
+        <f aca="false">IF($B22="","",IFERROR(ROUND(IF($C22="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B22),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B22,'Score Log'!$D$4:$D$203,$C22)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J22" s="40" t="str">
+        <f aca="false">IF(OR($B22="",$D22=0),"",IFERROR(IF($C22="",COUNTIFS('Score Log'!$C$4:$C$203,$B22,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B22,'Score Log'!$D$4:$D$203,$C22,'Score Log'!$U$4:$U$203,"Yes"))/$D22,"-"))</f>
         <v/>
       </c>
       <c r="K22" s="41" t="str">
-        <f aca="false">IF($A22="","",IF(AND(ISNUMBER($F22),ISNUMBER($C22)),MAX(1,MIN(5,ROUND(6-AVERAGE($F22,$C22),0))),IF(ISNUMBER($F22),MAX(1,MIN(5,ROUND(6-$F22,0))),"-")))</f>
+        <f aca="false">IF($B22="","",IF(ISNUMBER($F22),MAX(1,MIN(5,ROUND(6-$F22,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L22" s="41" t="str">
+        <f aca="false">IF($B22="","",IF(ISNUMBER($G22),MAX(1,MIN(5,ROUND(6-$G22,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M22" s="41" t="str">
+        <f aca="false">IF($B22="","",IF(AND(ISNUMBER($P22),ISNUMBER($O22)),MAX(1,MIN(5,ROUND(6-AVERAGE($P22,$O22),0))),IF(ISNUMBER($P22),MAX(1,MIN(5,ROUND(6-$P22,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O22" s="33" t="str">
+        <f aca="false">IF($B22="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B22),""))</f>
+        <v/>
+      </c>
+      <c r="P22" s="33" t="str">
+        <f aca="false">IF($B22="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B22),""))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="37" t="str">
-        <f aca="false">IF(Suppliers!A21="","",Suppliers!A21)</f>
-        <v/>
-      </c>
-      <c r="B23" s="38" t="str">
-        <f aca="false">IF($A23="","",COUNTIF('Score Log'!$C$4:$C$203,$A23))</f>
-        <v/>
-      </c>
-      <c r="C23" s="39" t="str">
-        <f aca="false">IF($A23="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A23),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D23" s="39" t="str">
-        <f aca="false">IF($A23="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A23),1),"-"))</f>
+      <c r="A23" s="37"/>
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="38" t="str">
+        <f aca="false">IF($B23="","",IF($C23="",COUNTIF('Score Log'!$C$4:$C$203,$B23),COUNTIFS('Score Log'!$C$4:$C$203,$B23,'Score Log'!$D$4:$D$203,$C23)))</f>
         <v/>
       </c>
       <c r="E23" s="39" t="str">
-        <f aca="false">IF($A23="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A23),1),"-"))</f>
+        <f aca="false">IF($B23="","",IFERROR(ROUND(IF($C23="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B23),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B23,'Score Log'!$D$4:$D$203,$C23)),1),"-"))</f>
         <v/>
       </c>
       <c r="F23" s="39" t="str">
-        <f aca="false">IF($A23="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A23),1),"-"))</f>
+        <f aca="false">IF($B23="","",IFERROR(ROUND(IF($C23="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B23),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B23,'Score Log'!$D$4:$D$203,$C23)),1),"-"))</f>
         <v/>
       </c>
       <c r="G23" s="39" t="str">
-        <f aca="false">IF($A23="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A23),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H23" s="40" t="str">
-        <f aca="false">IF($A23="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A23,'Score Log'!$U$4:$U$203,"Yes")/$B23,"-"))</f>
-        <v/>
-      </c>
-      <c r="I23" s="41" t="str">
-        <f aca="false">IF($A23="","",IF(ISNUMBER($D23),MAX(1,MIN(5,ROUND(6-$D23,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J23" s="41" t="str">
-        <f aca="false">IF($A23="","",IF(ISNUMBER($E23),MAX(1,MIN(5,ROUND(6-$E23,0))),"-"))</f>
+        <f aca="false">IF($B23="","",IFERROR(ROUND(IF($C23="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B23),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B23,'Score Log'!$D$4:$D$203,$C23)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H23" s="39" t="str">
+        <f aca="false">IF($B23="","",IFERROR(ROUND(IF($C23="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B23),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B23,'Score Log'!$D$4:$D$203,$C23)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I23" s="39" t="str">
+        <f aca="false">IF($B23="","",IFERROR(ROUND(IF($C23="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B23),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B23,'Score Log'!$D$4:$D$203,$C23)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J23" s="40" t="str">
+        <f aca="false">IF(OR($B23="",$D23=0),"",IFERROR(IF($C23="",COUNTIFS('Score Log'!$C$4:$C$203,$B23,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B23,'Score Log'!$D$4:$D$203,$C23,'Score Log'!$U$4:$U$203,"Yes"))/$D23,"-"))</f>
         <v/>
       </c>
       <c r="K23" s="41" t="str">
-        <f aca="false">IF($A23="","",IF(AND(ISNUMBER($F23),ISNUMBER($C23)),MAX(1,MIN(5,ROUND(6-AVERAGE($F23,$C23),0))),IF(ISNUMBER($F23),MAX(1,MIN(5,ROUND(6-$F23,0))),"-")))</f>
+        <f aca="false">IF($B23="","",IF(ISNUMBER($F23),MAX(1,MIN(5,ROUND(6-$F23,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L23" s="41" t="str">
+        <f aca="false">IF($B23="","",IF(ISNUMBER($G23),MAX(1,MIN(5,ROUND(6-$G23,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M23" s="41" t="str">
+        <f aca="false">IF($B23="","",IF(AND(ISNUMBER($P23),ISNUMBER($O23)),MAX(1,MIN(5,ROUND(6-AVERAGE($P23,$O23),0))),IF(ISNUMBER($P23),MAX(1,MIN(5,ROUND(6-$P23,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O23" s="33" t="str">
+        <f aca="false">IF($B23="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B23),""))</f>
+        <v/>
+      </c>
+      <c r="P23" s="33" t="str">
+        <f aca="false">IF($B23="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B23),""))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="37" t="str">
-        <f aca="false">IF(Suppliers!A22="","",Suppliers!A22)</f>
-        <v/>
-      </c>
-      <c r="B24" s="38" t="str">
-        <f aca="false">IF($A24="","",COUNTIF('Score Log'!$C$4:$C$203,$A24))</f>
-        <v/>
-      </c>
-      <c r="C24" s="39" t="str">
-        <f aca="false">IF($A24="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A24),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D24" s="39" t="str">
-        <f aca="false">IF($A24="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A24),1),"-"))</f>
+      <c r="A24" s="37"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="38" t="str">
+        <f aca="false">IF($B24="","",IF($C24="",COUNTIF('Score Log'!$C$4:$C$203,$B24),COUNTIFS('Score Log'!$C$4:$C$203,$B24,'Score Log'!$D$4:$D$203,$C24)))</f>
         <v/>
       </c>
       <c r="E24" s="39" t="str">
-        <f aca="false">IF($A24="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A24),1),"-"))</f>
+        <f aca="false">IF($B24="","",IFERROR(ROUND(IF($C24="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B24),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B24,'Score Log'!$D$4:$D$203,$C24)),1),"-"))</f>
         <v/>
       </c>
       <c r="F24" s="39" t="str">
-        <f aca="false">IF($A24="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A24),1),"-"))</f>
+        <f aca="false">IF($B24="","",IFERROR(ROUND(IF($C24="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B24),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B24,'Score Log'!$D$4:$D$203,$C24)),1),"-"))</f>
         <v/>
       </c>
       <c r="G24" s="39" t="str">
-        <f aca="false">IF($A24="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A24),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H24" s="40" t="str">
-        <f aca="false">IF($A24="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A24,'Score Log'!$U$4:$U$203,"Yes")/$B24,"-"))</f>
-        <v/>
-      </c>
-      <c r="I24" s="41" t="str">
-        <f aca="false">IF($A24="","",IF(ISNUMBER($D24),MAX(1,MIN(5,ROUND(6-$D24,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J24" s="41" t="str">
-        <f aca="false">IF($A24="","",IF(ISNUMBER($E24),MAX(1,MIN(5,ROUND(6-$E24,0))),"-"))</f>
+        <f aca="false">IF($B24="","",IFERROR(ROUND(IF($C24="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B24),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B24,'Score Log'!$D$4:$D$203,$C24)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H24" s="39" t="str">
+        <f aca="false">IF($B24="","",IFERROR(ROUND(IF($C24="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B24),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B24,'Score Log'!$D$4:$D$203,$C24)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I24" s="39" t="str">
+        <f aca="false">IF($B24="","",IFERROR(ROUND(IF($C24="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B24),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B24,'Score Log'!$D$4:$D$203,$C24)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J24" s="40" t="str">
+        <f aca="false">IF(OR($B24="",$D24=0),"",IFERROR(IF($C24="",COUNTIFS('Score Log'!$C$4:$C$203,$B24,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B24,'Score Log'!$D$4:$D$203,$C24,'Score Log'!$U$4:$U$203,"Yes"))/$D24,"-"))</f>
         <v/>
       </c>
       <c r="K24" s="41" t="str">
-        <f aca="false">IF($A24="","",IF(AND(ISNUMBER($F24),ISNUMBER($C24)),MAX(1,MIN(5,ROUND(6-AVERAGE($F24,$C24),0))),IF(ISNUMBER($F24),MAX(1,MIN(5,ROUND(6-$F24,0))),"-")))</f>
+        <f aca="false">IF($B24="","",IF(ISNUMBER($F24),MAX(1,MIN(5,ROUND(6-$F24,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L24" s="41" t="str">
+        <f aca="false">IF($B24="","",IF(ISNUMBER($G24),MAX(1,MIN(5,ROUND(6-$G24,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M24" s="41" t="str">
+        <f aca="false">IF($B24="","",IF(AND(ISNUMBER($P24),ISNUMBER($O24)),MAX(1,MIN(5,ROUND(6-AVERAGE($P24,$O24),0))),IF(ISNUMBER($P24),MAX(1,MIN(5,ROUND(6-$P24,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O24" s="33" t="str">
+        <f aca="false">IF($B24="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B24),""))</f>
+        <v/>
+      </c>
+      <c r="P24" s="33" t="str">
+        <f aca="false">IF($B24="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B24),""))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="37" t="str">
-        <f aca="false">IF(Suppliers!A23="","",Suppliers!A23)</f>
-        <v/>
-      </c>
-      <c r="B25" s="38" t="str">
-        <f aca="false">IF($A25="","",COUNTIF('Score Log'!$C$4:$C$203,$A25))</f>
-        <v/>
-      </c>
-      <c r="C25" s="39" t="str">
-        <f aca="false">IF($A25="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A25),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D25" s="39" t="str">
-        <f aca="false">IF($A25="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A25),1),"-"))</f>
+      <c r="A25" s="37"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="38" t="str">
+        <f aca="false">IF($B25="","",IF($C25="",COUNTIF('Score Log'!$C$4:$C$203,$B25),COUNTIFS('Score Log'!$C$4:$C$203,$B25,'Score Log'!$D$4:$D$203,$C25)))</f>
         <v/>
       </c>
       <c r="E25" s="39" t="str">
-        <f aca="false">IF($A25="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A25),1),"-"))</f>
+        <f aca="false">IF($B25="","",IFERROR(ROUND(IF($C25="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B25),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B25,'Score Log'!$D$4:$D$203,$C25)),1),"-"))</f>
         <v/>
       </c>
       <c r="F25" s="39" t="str">
-        <f aca="false">IF($A25="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A25),1),"-"))</f>
+        <f aca="false">IF($B25="","",IFERROR(ROUND(IF($C25="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B25),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B25,'Score Log'!$D$4:$D$203,$C25)),1),"-"))</f>
         <v/>
       </c>
       <c r="G25" s="39" t="str">
-        <f aca="false">IF($A25="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A25),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H25" s="40" t="str">
-        <f aca="false">IF($A25="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A25,'Score Log'!$U$4:$U$203,"Yes")/$B25,"-"))</f>
-        <v/>
-      </c>
-      <c r="I25" s="41" t="str">
-        <f aca="false">IF($A25="","",IF(ISNUMBER($D25),MAX(1,MIN(5,ROUND(6-$D25,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J25" s="41" t="str">
-        <f aca="false">IF($A25="","",IF(ISNUMBER($E25),MAX(1,MIN(5,ROUND(6-$E25,0))),"-"))</f>
+        <f aca="false">IF($B25="","",IFERROR(ROUND(IF($C25="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B25),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B25,'Score Log'!$D$4:$D$203,$C25)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H25" s="39" t="str">
+        <f aca="false">IF($B25="","",IFERROR(ROUND(IF($C25="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B25),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B25,'Score Log'!$D$4:$D$203,$C25)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I25" s="39" t="str">
+        <f aca="false">IF($B25="","",IFERROR(ROUND(IF($C25="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B25),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B25,'Score Log'!$D$4:$D$203,$C25)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J25" s="40" t="str">
+        <f aca="false">IF(OR($B25="",$D25=0),"",IFERROR(IF($C25="",COUNTIFS('Score Log'!$C$4:$C$203,$B25,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B25,'Score Log'!$D$4:$D$203,$C25,'Score Log'!$U$4:$U$203,"Yes"))/$D25,"-"))</f>
         <v/>
       </c>
       <c r="K25" s="41" t="str">
-        <f aca="false">IF($A25="","",IF(AND(ISNUMBER($F25),ISNUMBER($C25)),MAX(1,MIN(5,ROUND(6-AVERAGE($F25,$C25),0))),IF(ISNUMBER($F25),MAX(1,MIN(5,ROUND(6-$F25,0))),"-")))</f>
+        <f aca="false">IF($B25="","",IF(ISNUMBER($F25),MAX(1,MIN(5,ROUND(6-$F25,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L25" s="41" t="str">
+        <f aca="false">IF($B25="","",IF(ISNUMBER($G25),MAX(1,MIN(5,ROUND(6-$G25,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M25" s="41" t="str">
+        <f aca="false">IF($B25="","",IF(AND(ISNUMBER($P25),ISNUMBER($O25)),MAX(1,MIN(5,ROUND(6-AVERAGE($P25,$O25),0))),IF(ISNUMBER($P25),MAX(1,MIN(5,ROUND(6-$P25,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O25" s="33" t="str">
+        <f aca="false">IF($B25="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B25),""))</f>
+        <v/>
+      </c>
+      <c r="P25" s="33" t="str">
+        <f aca="false">IF($B25="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B25),""))</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="37" t="str">
-        <f aca="false">IF(Suppliers!A24="","",Suppliers!A24)</f>
-        <v/>
-      </c>
-      <c r="B26" s="38" t="str">
-        <f aca="false">IF($A26="","",COUNTIF('Score Log'!$C$4:$C$203,$A26))</f>
-        <v/>
-      </c>
-      <c r="C26" s="39" t="str">
-        <f aca="false">IF($A26="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A26),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D26" s="39" t="str">
-        <f aca="false">IF($A26="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A26),1),"-"))</f>
+      <c r="A26" s="37"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="38" t="str">
+        <f aca="false">IF($B26="","",IF($C26="",COUNTIF('Score Log'!$C$4:$C$203,$B26),COUNTIFS('Score Log'!$C$4:$C$203,$B26,'Score Log'!$D$4:$D$203,$C26)))</f>
         <v/>
       </c>
       <c r="E26" s="39" t="str">
-        <f aca="false">IF($A26="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A26),1),"-"))</f>
+        <f aca="false">IF($B26="","",IFERROR(ROUND(IF($C26="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B26),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B26,'Score Log'!$D$4:$D$203,$C26)),1),"-"))</f>
         <v/>
       </c>
       <c r="F26" s="39" t="str">
-        <f aca="false">IF($A26="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A26),1),"-"))</f>
+        <f aca="false">IF($B26="","",IFERROR(ROUND(IF($C26="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B26),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B26,'Score Log'!$D$4:$D$203,$C26)),1),"-"))</f>
         <v/>
       </c>
       <c r="G26" s="39" t="str">
-        <f aca="false">IF($A26="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A26),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H26" s="40" t="str">
-        <f aca="false">IF($A26="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A26,'Score Log'!$U$4:$U$203,"Yes")/$B26,"-"))</f>
-        <v/>
-      </c>
-      <c r="I26" s="41" t="str">
-        <f aca="false">IF($A26="","",IF(ISNUMBER($D26),MAX(1,MIN(5,ROUND(6-$D26,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J26" s="41" t="str">
-        <f aca="false">IF($A26="","",IF(ISNUMBER($E26),MAX(1,MIN(5,ROUND(6-$E26,0))),"-"))</f>
+        <f aca="false">IF($B26="","",IFERROR(ROUND(IF($C26="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B26),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B26,'Score Log'!$D$4:$D$203,$C26)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H26" s="39" t="str">
+        <f aca="false">IF($B26="","",IFERROR(ROUND(IF($C26="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B26),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B26,'Score Log'!$D$4:$D$203,$C26)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I26" s="39" t="str">
+        <f aca="false">IF($B26="","",IFERROR(ROUND(IF($C26="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B26),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B26,'Score Log'!$D$4:$D$203,$C26)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J26" s="40" t="str">
+        <f aca="false">IF(OR($B26="",$D26=0),"",IFERROR(IF($C26="",COUNTIFS('Score Log'!$C$4:$C$203,$B26,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B26,'Score Log'!$D$4:$D$203,$C26,'Score Log'!$U$4:$U$203,"Yes"))/$D26,"-"))</f>
         <v/>
       </c>
       <c r="K26" s="41" t="str">
-        <f aca="false">IF($A26="","",IF(AND(ISNUMBER($F26),ISNUMBER($C26)),MAX(1,MIN(5,ROUND(6-AVERAGE($F26,$C26),0))),IF(ISNUMBER($F26),MAX(1,MIN(5,ROUND(6-$F26,0))),"-")))</f>
+        <f aca="false">IF($B26="","",IF(ISNUMBER($F26),MAX(1,MIN(5,ROUND(6-$F26,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L26" s="41" t="str">
+        <f aca="false">IF($B26="","",IF(ISNUMBER($G26),MAX(1,MIN(5,ROUND(6-$G26,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M26" s="41" t="str">
+        <f aca="false">IF($B26="","",IF(AND(ISNUMBER($P26),ISNUMBER($O26)),MAX(1,MIN(5,ROUND(6-AVERAGE($P26,$O26),0))),IF(ISNUMBER($P26),MAX(1,MIN(5,ROUND(6-$P26,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O26" s="33" t="str">
+        <f aca="false">IF($B26="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B26),""))</f>
+        <v/>
+      </c>
+      <c r="P26" s="33" t="str">
+        <f aca="false">IF($B26="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B26),""))</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="37" t="str">
-        <f aca="false">IF(Suppliers!A25="","",Suppliers!A25)</f>
-        <v/>
-      </c>
-      <c r="B27" s="38" t="str">
-        <f aca="false">IF($A27="","",COUNTIF('Score Log'!$C$4:$C$203,$A27))</f>
-        <v/>
-      </c>
-      <c r="C27" s="39" t="str">
-        <f aca="false">IF($A27="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A27),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D27" s="39" t="str">
-        <f aca="false">IF($A27="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A27),1),"-"))</f>
+      <c r="A27" s="37"/>
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="38" t="str">
+        <f aca="false">IF($B27="","",IF($C27="",COUNTIF('Score Log'!$C$4:$C$203,$B27),COUNTIFS('Score Log'!$C$4:$C$203,$B27,'Score Log'!$D$4:$D$203,$C27)))</f>
         <v/>
       </c>
       <c r="E27" s="39" t="str">
-        <f aca="false">IF($A27="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A27),1),"-"))</f>
+        <f aca="false">IF($B27="","",IFERROR(ROUND(IF($C27="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B27),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B27,'Score Log'!$D$4:$D$203,$C27)),1),"-"))</f>
         <v/>
       </c>
       <c r="F27" s="39" t="str">
-        <f aca="false">IF($A27="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A27),1),"-"))</f>
+        <f aca="false">IF($B27="","",IFERROR(ROUND(IF($C27="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B27),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B27,'Score Log'!$D$4:$D$203,$C27)),1),"-"))</f>
         <v/>
       </c>
       <c r="G27" s="39" t="str">
-        <f aca="false">IF($A27="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A27),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H27" s="40" t="str">
-        <f aca="false">IF($A27="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A27,'Score Log'!$U$4:$U$203,"Yes")/$B27,"-"))</f>
-        <v/>
-      </c>
-      <c r="I27" s="41" t="str">
-        <f aca="false">IF($A27="","",IF(ISNUMBER($D27),MAX(1,MIN(5,ROUND(6-$D27,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J27" s="41" t="str">
-        <f aca="false">IF($A27="","",IF(ISNUMBER($E27),MAX(1,MIN(5,ROUND(6-$E27,0))),"-"))</f>
+        <f aca="false">IF($B27="","",IFERROR(ROUND(IF($C27="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B27),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B27,'Score Log'!$D$4:$D$203,$C27)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H27" s="39" t="str">
+        <f aca="false">IF($B27="","",IFERROR(ROUND(IF($C27="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B27),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B27,'Score Log'!$D$4:$D$203,$C27)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I27" s="39" t="str">
+        <f aca="false">IF($B27="","",IFERROR(ROUND(IF($C27="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B27),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B27,'Score Log'!$D$4:$D$203,$C27)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J27" s="40" t="str">
+        <f aca="false">IF(OR($B27="",$D27=0),"",IFERROR(IF($C27="",COUNTIFS('Score Log'!$C$4:$C$203,$B27,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B27,'Score Log'!$D$4:$D$203,$C27,'Score Log'!$U$4:$U$203,"Yes"))/$D27,"-"))</f>
         <v/>
       </c>
       <c r="K27" s="41" t="str">
-        <f aca="false">IF($A27="","",IF(AND(ISNUMBER($F27),ISNUMBER($C27)),MAX(1,MIN(5,ROUND(6-AVERAGE($F27,$C27),0))),IF(ISNUMBER($F27),MAX(1,MIN(5,ROUND(6-$F27,0))),"-")))</f>
+        <f aca="false">IF($B27="","",IF(ISNUMBER($F27),MAX(1,MIN(5,ROUND(6-$F27,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L27" s="41" t="str">
+        <f aca="false">IF($B27="","",IF(ISNUMBER($G27),MAX(1,MIN(5,ROUND(6-$G27,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M27" s="41" t="str">
+        <f aca="false">IF($B27="","",IF(AND(ISNUMBER($P27),ISNUMBER($O27)),MAX(1,MIN(5,ROUND(6-AVERAGE($P27,$O27),0))),IF(ISNUMBER($P27),MAX(1,MIN(5,ROUND(6-$P27,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O27" s="33" t="str">
+        <f aca="false">IF($B27="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B27),""))</f>
+        <v/>
+      </c>
+      <c r="P27" s="33" t="str">
+        <f aca="false">IF($B27="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B27),""))</f>
         <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="37" t="str">
-        <f aca="false">IF(Suppliers!A26="","",Suppliers!A26)</f>
-        <v/>
-      </c>
-      <c r="B28" s="38" t="str">
-        <f aca="false">IF($A28="","",COUNTIF('Score Log'!$C$4:$C$203,$A28))</f>
-        <v/>
-      </c>
-      <c r="C28" s="39" t="str">
-        <f aca="false">IF($A28="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A28),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D28" s="39" t="str">
-        <f aca="false">IF($A28="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A28),1),"-"))</f>
+      <c r="A28" s="37"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="38" t="str">
+        <f aca="false">IF($B28="","",IF($C28="",COUNTIF('Score Log'!$C$4:$C$203,$B28),COUNTIFS('Score Log'!$C$4:$C$203,$B28,'Score Log'!$D$4:$D$203,$C28)))</f>
         <v/>
       </c>
       <c r="E28" s="39" t="str">
-        <f aca="false">IF($A28="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A28),1),"-"))</f>
+        <f aca="false">IF($B28="","",IFERROR(ROUND(IF($C28="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B28),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B28,'Score Log'!$D$4:$D$203,$C28)),1),"-"))</f>
         <v/>
       </c>
       <c r="F28" s="39" t="str">
-        <f aca="false">IF($A28="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A28),1),"-"))</f>
+        <f aca="false">IF($B28="","",IFERROR(ROUND(IF($C28="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B28),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B28,'Score Log'!$D$4:$D$203,$C28)),1),"-"))</f>
         <v/>
       </c>
       <c r="G28" s="39" t="str">
-        <f aca="false">IF($A28="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A28),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H28" s="40" t="str">
-        <f aca="false">IF($A28="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A28,'Score Log'!$U$4:$U$203,"Yes")/$B28,"-"))</f>
-        <v/>
-      </c>
-      <c r="I28" s="41" t="str">
-        <f aca="false">IF($A28="","",IF(ISNUMBER($D28),MAX(1,MIN(5,ROUND(6-$D28,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J28" s="41" t="str">
-        <f aca="false">IF($A28="","",IF(ISNUMBER($E28),MAX(1,MIN(5,ROUND(6-$E28,0))),"-"))</f>
+        <f aca="false">IF($B28="","",IFERROR(ROUND(IF($C28="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B28),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B28,'Score Log'!$D$4:$D$203,$C28)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H28" s="39" t="str">
+        <f aca="false">IF($B28="","",IFERROR(ROUND(IF($C28="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B28),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B28,'Score Log'!$D$4:$D$203,$C28)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I28" s="39" t="str">
+        <f aca="false">IF($B28="","",IFERROR(ROUND(IF($C28="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B28),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B28,'Score Log'!$D$4:$D$203,$C28)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J28" s="40" t="str">
+        <f aca="false">IF(OR($B28="",$D28=0),"",IFERROR(IF($C28="",COUNTIFS('Score Log'!$C$4:$C$203,$B28,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B28,'Score Log'!$D$4:$D$203,$C28,'Score Log'!$U$4:$U$203,"Yes"))/$D28,"-"))</f>
         <v/>
       </c>
       <c r="K28" s="41" t="str">
-        <f aca="false">IF($A28="","",IF(AND(ISNUMBER($F28),ISNUMBER($C28)),MAX(1,MIN(5,ROUND(6-AVERAGE($F28,$C28),0))),IF(ISNUMBER($F28),MAX(1,MIN(5,ROUND(6-$F28,0))),"-")))</f>
+        <f aca="false">IF($B28="","",IF(ISNUMBER($F28),MAX(1,MIN(5,ROUND(6-$F28,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L28" s="41" t="str">
+        <f aca="false">IF($B28="","",IF(ISNUMBER($G28),MAX(1,MIN(5,ROUND(6-$G28,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M28" s="41" t="str">
+        <f aca="false">IF($B28="","",IF(AND(ISNUMBER($P28),ISNUMBER($O28)),MAX(1,MIN(5,ROUND(6-AVERAGE($P28,$O28),0))),IF(ISNUMBER($P28),MAX(1,MIN(5,ROUND(6-$P28,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O28" s="33" t="str">
+        <f aca="false">IF($B28="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B28),""))</f>
+        <v/>
+      </c>
+      <c r="P28" s="33" t="str">
+        <f aca="false">IF($B28="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B28),""))</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="37" t="str">
-        <f aca="false">IF(Suppliers!A27="","",Suppliers!A27)</f>
-        <v/>
-      </c>
-      <c r="B29" s="38" t="str">
-        <f aca="false">IF($A29="","",COUNTIF('Score Log'!$C$4:$C$203,$A29))</f>
-        <v/>
-      </c>
-      <c r="C29" s="39" t="str">
-        <f aca="false">IF($A29="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A29),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D29" s="39" t="str">
-        <f aca="false">IF($A29="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A29),1),"-"))</f>
+      <c r="A29" s="37"/>
+      <c r="B29" s="37"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="38" t="str">
+        <f aca="false">IF($B29="","",IF($C29="",COUNTIF('Score Log'!$C$4:$C$203,$B29),COUNTIFS('Score Log'!$C$4:$C$203,$B29,'Score Log'!$D$4:$D$203,$C29)))</f>
         <v/>
       </c>
       <c r="E29" s="39" t="str">
-        <f aca="false">IF($A29="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A29),1),"-"))</f>
+        <f aca="false">IF($B29="","",IFERROR(ROUND(IF($C29="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B29),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B29,'Score Log'!$D$4:$D$203,$C29)),1),"-"))</f>
         <v/>
       </c>
       <c r="F29" s="39" t="str">
-        <f aca="false">IF($A29="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A29),1),"-"))</f>
+        <f aca="false">IF($B29="","",IFERROR(ROUND(IF($C29="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B29),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B29,'Score Log'!$D$4:$D$203,$C29)),1),"-"))</f>
         <v/>
       </c>
       <c r="G29" s="39" t="str">
-        <f aca="false">IF($A29="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A29),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H29" s="40" t="str">
-        <f aca="false">IF($A29="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A29,'Score Log'!$U$4:$U$203,"Yes")/$B29,"-"))</f>
-        <v/>
-      </c>
-      <c r="I29" s="41" t="str">
-        <f aca="false">IF($A29="","",IF(ISNUMBER($D29),MAX(1,MIN(5,ROUND(6-$D29,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J29" s="41" t="str">
-        <f aca="false">IF($A29="","",IF(ISNUMBER($E29),MAX(1,MIN(5,ROUND(6-$E29,0))),"-"))</f>
+        <f aca="false">IF($B29="","",IFERROR(ROUND(IF($C29="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B29),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B29,'Score Log'!$D$4:$D$203,$C29)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H29" s="39" t="str">
+        <f aca="false">IF($B29="","",IFERROR(ROUND(IF($C29="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B29),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B29,'Score Log'!$D$4:$D$203,$C29)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I29" s="39" t="str">
+        <f aca="false">IF($B29="","",IFERROR(ROUND(IF($C29="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B29),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B29,'Score Log'!$D$4:$D$203,$C29)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J29" s="40" t="str">
+        <f aca="false">IF(OR($B29="",$D29=0),"",IFERROR(IF($C29="",COUNTIFS('Score Log'!$C$4:$C$203,$B29,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B29,'Score Log'!$D$4:$D$203,$C29,'Score Log'!$U$4:$U$203,"Yes"))/$D29,"-"))</f>
         <v/>
       </c>
       <c r="K29" s="41" t="str">
-        <f aca="false">IF($A29="","",IF(AND(ISNUMBER($F29),ISNUMBER($C29)),MAX(1,MIN(5,ROUND(6-AVERAGE($F29,$C29),0))),IF(ISNUMBER($F29),MAX(1,MIN(5,ROUND(6-$F29,0))),"-")))</f>
+        <f aca="false">IF($B29="","",IF(ISNUMBER($F29),MAX(1,MIN(5,ROUND(6-$F29,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L29" s="41" t="str">
+        <f aca="false">IF($B29="","",IF(ISNUMBER($G29),MAX(1,MIN(5,ROUND(6-$G29,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M29" s="41" t="str">
+        <f aca="false">IF($B29="","",IF(AND(ISNUMBER($P29),ISNUMBER($O29)),MAX(1,MIN(5,ROUND(6-AVERAGE($P29,$O29),0))),IF(ISNUMBER($P29),MAX(1,MIN(5,ROUND(6-$P29,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O29" s="33" t="str">
+        <f aca="false">IF($B29="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B29),""))</f>
+        <v/>
+      </c>
+      <c r="P29" s="33" t="str">
+        <f aca="false">IF($B29="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B29),""))</f>
         <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="37" t="str">
-        <f aca="false">IF(Suppliers!A28="","",Suppliers!A28)</f>
-        <v/>
-      </c>
-      <c r="B30" s="38" t="str">
-        <f aca="false">IF($A30="","",COUNTIF('Score Log'!$C$4:$C$203,$A30))</f>
-        <v/>
-      </c>
-      <c r="C30" s="39" t="str">
-        <f aca="false">IF($A30="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A30),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D30" s="39" t="str">
-        <f aca="false">IF($A30="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A30),1),"-"))</f>
+      <c r="A30" s="37"/>
+      <c r="B30" s="37"/>
+      <c r="C30" s="37"/>
+      <c r="D30" s="38" t="str">
+        <f aca="false">IF($B30="","",IF($C30="",COUNTIF('Score Log'!$C$4:$C$203,$B30),COUNTIFS('Score Log'!$C$4:$C$203,$B30,'Score Log'!$D$4:$D$203,$C30)))</f>
         <v/>
       </c>
       <c r="E30" s="39" t="str">
-        <f aca="false">IF($A30="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A30),1),"-"))</f>
+        <f aca="false">IF($B30="","",IFERROR(ROUND(IF($C30="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B30),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B30,'Score Log'!$D$4:$D$203,$C30)),1),"-"))</f>
         <v/>
       </c>
       <c r="F30" s="39" t="str">
-        <f aca="false">IF($A30="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A30),1),"-"))</f>
+        <f aca="false">IF($B30="","",IFERROR(ROUND(IF($C30="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B30),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B30,'Score Log'!$D$4:$D$203,$C30)),1),"-"))</f>
         <v/>
       </c>
       <c r="G30" s="39" t="str">
-        <f aca="false">IF($A30="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A30),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H30" s="40" t="str">
-        <f aca="false">IF($A30="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A30,'Score Log'!$U$4:$U$203,"Yes")/$B30,"-"))</f>
-        <v/>
-      </c>
-      <c r="I30" s="41" t="str">
-        <f aca="false">IF($A30="","",IF(ISNUMBER($D30),MAX(1,MIN(5,ROUND(6-$D30,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J30" s="41" t="str">
-        <f aca="false">IF($A30="","",IF(ISNUMBER($E30),MAX(1,MIN(5,ROUND(6-$E30,0))),"-"))</f>
+        <f aca="false">IF($B30="","",IFERROR(ROUND(IF($C30="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B30),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B30,'Score Log'!$D$4:$D$203,$C30)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H30" s="39" t="str">
+        <f aca="false">IF($B30="","",IFERROR(ROUND(IF($C30="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B30),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B30,'Score Log'!$D$4:$D$203,$C30)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I30" s="39" t="str">
+        <f aca="false">IF($B30="","",IFERROR(ROUND(IF($C30="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B30),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B30,'Score Log'!$D$4:$D$203,$C30)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J30" s="40" t="str">
+        <f aca="false">IF(OR($B30="",$D30=0),"",IFERROR(IF($C30="",COUNTIFS('Score Log'!$C$4:$C$203,$B30,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B30,'Score Log'!$D$4:$D$203,$C30,'Score Log'!$U$4:$U$203,"Yes"))/$D30,"-"))</f>
         <v/>
       </c>
       <c r="K30" s="41" t="str">
-        <f aca="false">IF($A30="","",IF(AND(ISNUMBER($F30),ISNUMBER($C30)),MAX(1,MIN(5,ROUND(6-AVERAGE($F30,$C30),0))),IF(ISNUMBER($F30),MAX(1,MIN(5,ROUND(6-$F30,0))),"-")))</f>
+        <f aca="false">IF($B30="","",IF(ISNUMBER($F30),MAX(1,MIN(5,ROUND(6-$F30,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L30" s="41" t="str">
+        <f aca="false">IF($B30="","",IF(ISNUMBER($G30),MAX(1,MIN(5,ROUND(6-$G30,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M30" s="41" t="str">
+        <f aca="false">IF($B30="","",IF(AND(ISNUMBER($P30),ISNUMBER($O30)),MAX(1,MIN(5,ROUND(6-AVERAGE($P30,$O30),0))),IF(ISNUMBER($P30),MAX(1,MIN(5,ROUND(6-$P30,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O30" s="33" t="str">
+        <f aca="false">IF($B30="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B30),""))</f>
+        <v/>
+      </c>
+      <c r="P30" s="33" t="str">
+        <f aca="false">IF($B30="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B30),""))</f>
         <v/>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="37" t="str">
-        <f aca="false">IF(Suppliers!A29="","",Suppliers!A29)</f>
-        <v/>
-      </c>
-      <c r="B31" s="38" t="str">
-        <f aca="false">IF($A31="","",COUNTIF('Score Log'!$C$4:$C$203,$A31))</f>
-        <v/>
-      </c>
-      <c r="C31" s="39" t="str">
-        <f aca="false">IF($A31="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A31),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D31" s="39" t="str">
-        <f aca="false">IF($A31="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A31),1),"-"))</f>
+      <c r="A31" s="37"/>
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="38" t="str">
+        <f aca="false">IF($B31="","",IF($C31="",COUNTIF('Score Log'!$C$4:$C$203,$B31),COUNTIFS('Score Log'!$C$4:$C$203,$B31,'Score Log'!$D$4:$D$203,$C31)))</f>
         <v/>
       </c>
       <c r="E31" s="39" t="str">
-        <f aca="false">IF($A31="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A31),1),"-"))</f>
+        <f aca="false">IF($B31="","",IFERROR(ROUND(IF($C31="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B31),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B31,'Score Log'!$D$4:$D$203,$C31)),1),"-"))</f>
         <v/>
       </c>
       <c r="F31" s="39" t="str">
-        <f aca="false">IF($A31="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A31),1),"-"))</f>
+        <f aca="false">IF($B31="","",IFERROR(ROUND(IF($C31="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B31),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B31,'Score Log'!$D$4:$D$203,$C31)),1),"-"))</f>
         <v/>
       </c>
       <c r="G31" s="39" t="str">
-        <f aca="false">IF($A31="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A31),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H31" s="40" t="str">
-        <f aca="false">IF($A31="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A31,'Score Log'!$U$4:$U$203,"Yes")/$B31,"-"))</f>
-        <v/>
-      </c>
-      <c r="I31" s="41" t="str">
-        <f aca="false">IF($A31="","",IF(ISNUMBER($D31),MAX(1,MIN(5,ROUND(6-$D31,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J31" s="41" t="str">
-        <f aca="false">IF($A31="","",IF(ISNUMBER($E31),MAX(1,MIN(5,ROUND(6-$E31,0))),"-"))</f>
+        <f aca="false">IF($B31="","",IFERROR(ROUND(IF($C31="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B31),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B31,'Score Log'!$D$4:$D$203,$C31)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H31" s="39" t="str">
+        <f aca="false">IF($B31="","",IFERROR(ROUND(IF($C31="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B31),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B31,'Score Log'!$D$4:$D$203,$C31)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I31" s="39" t="str">
+        <f aca="false">IF($B31="","",IFERROR(ROUND(IF($C31="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B31),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B31,'Score Log'!$D$4:$D$203,$C31)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J31" s="40" t="str">
+        <f aca="false">IF(OR($B31="",$D31=0),"",IFERROR(IF($C31="",COUNTIFS('Score Log'!$C$4:$C$203,$B31,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B31,'Score Log'!$D$4:$D$203,$C31,'Score Log'!$U$4:$U$203,"Yes"))/$D31,"-"))</f>
         <v/>
       </c>
       <c r="K31" s="41" t="str">
-        <f aca="false">IF($A31="","",IF(AND(ISNUMBER($F31),ISNUMBER($C31)),MAX(1,MIN(5,ROUND(6-AVERAGE($F31,$C31),0))),IF(ISNUMBER($F31),MAX(1,MIN(5,ROUND(6-$F31,0))),"-")))</f>
+        <f aca="false">IF($B31="","",IF(ISNUMBER($F31),MAX(1,MIN(5,ROUND(6-$F31,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L31" s="41" t="str">
+        <f aca="false">IF($B31="","",IF(ISNUMBER($G31),MAX(1,MIN(5,ROUND(6-$G31,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M31" s="41" t="str">
+        <f aca="false">IF($B31="","",IF(AND(ISNUMBER($P31),ISNUMBER($O31)),MAX(1,MIN(5,ROUND(6-AVERAGE($P31,$O31),0))),IF(ISNUMBER($P31),MAX(1,MIN(5,ROUND(6-$P31,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O31" s="33" t="str">
+        <f aca="false">IF($B31="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B31),""))</f>
+        <v/>
+      </c>
+      <c r="P31" s="33" t="str">
+        <f aca="false">IF($B31="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B31),""))</f>
         <v/>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="37" t="str">
-        <f aca="false">IF(Suppliers!A30="","",Suppliers!A30)</f>
-        <v/>
-      </c>
-      <c r="B32" s="38" t="str">
-        <f aca="false">IF($A32="","",COUNTIF('Score Log'!$C$4:$C$203,$A32))</f>
-        <v/>
-      </c>
-      <c r="C32" s="39" t="str">
-        <f aca="false">IF($A32="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A32),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D32" s="39" t="str">
-        <f aca="false">IF($A32="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A32),1),"-"))</f>
+      <c r="A32" s="37"/>
+      <c r="B32" s="37"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="38" t="str">
+        <f aca="false">IF($B32="","",IF($C32="",COUNTIF('Score Log'!$C$4:$C$203,$B32),COUNTIFS('Score Log'!$C$4:$C$203,$B32,'Score Log'!$D$4:$D$203,$C32)))</f>
         <v/>
       </c>
       <c r="E32" s="39" t="str">
-        <f aca="false">IF($A32="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A32),1),"-"))</f>
+        <f aca="false">IF($B32="","",IFERROR(ROUND(IF($C32="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B32),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B32,'Score Log'!$D$4:$D$203,$C32)),1),"-"))</f>
         <v/>
       </c>
       <c r="F32" s="39" t="str">
-        <f aca="false">IF($A32="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A32),1),"-"))</f>
+        <f aca="false">IF($B32="","",IFERROR(ROUND(IF($C32="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B32),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B32,'Score Log'!$D$4:$D$203,$C32)),1),"-"))</f>
         <v/>
       </c>
       <c r="G32" s="39" t="str">
-        <f aca="false">IF($A32="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A32),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H32" s="40" t="str">
-        <f aca="false">IF($A32="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A32,'Score Log'!$U$4:$U$203,"Yes")/$B32,"-"))</f>
-        <v/>
-      </c>
-      <c r="I32" s="41" t="str">
-        <f aca="false">IF($A32="","",IF(ISNUMBER($D32),MAX(1,MIN(5,ROUND(6-$D32,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J32" s="41" t="str">
-        <f aca="false">IF($A32="","",IF(ISNUMBER($E32),MAX(1,MIN(5,ROUND(6-$E32,0))),"-"))</f>
+        <f aca="false">IF($B32="","",IFERROR(ROUND(IF($C32="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B32),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B32,'Score Log'!$D$4:$D$203,$C32)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H32" s="39" t="str">
+        <f aca="false">IF($B32="","",IFERROR(ROUND(IF($C32="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B32),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B32,'Score Log'!$D$4:$D$203,$C32)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I32" s="39" t="str">
+        <f aca="false">IF($B32="","",IFERROR(ROUND(IF($C32="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B32),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B32,'Score Log'!$D$4:$D$203,$C32)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J32" s="40" t="str">
+        <f aca="false">IF(OR($B32="",$D32=0),"",IFERROR(IF($C32="",COUNTIFS('Score Log'!$C$4:$C$203,$B32,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B32,'Score Log'!$D$4:$D$203,$C32,'Score Log'!$U$4:$U$203,"Yes"))/$D32,"-"))</f>
         <v/>
       </c>
       <c r="K32" s="41" t="str">
-        <f aca="false">IF($A32="","",IF(AND(ISNUMBER($F32),ISNUMBER($C32)),MAX(1,MIN(5,ROUND(6-AVERAGE($F32,$C32),0))),IF(ISNUMBER($F32),MAX(1,MIN(5,ROUND(6-$F32,0))),"-")))</f>
+        <f aca="false">IF($B32="","",IF(ISNUMBER($F32),MAX(1,MIN(5,ROUND(6-$F32,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L32" s="41" t="str">
+        <f aca="false">IF($B32="","",IF(ISNUMBER($G32),MAX(1,MIN(5,ROUND(6-$G32,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M32" s="41" t="str">
+        <f aca="false">IF($B32="","",IF(AND(ISNUMBER($P32),ISNUMBER($O32)),MAX(1,MIN(5,ROUND(6-AVERAGE($P32,$O32),0))),IF(ISNUMBER($P32),MAX(1,MIN(5,ROUND(6-$P32,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O32" s="33" t="str">
+        <f aca="false">IF($B32="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B32),""))</f>
+        <v/>
+      </c>
+      <c r="P32" s="33" t="str">
+        <f aca="false">IF($B32="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B32),""))</f>
         <v/>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="37" t="str">
-        <f aca="false">IF(Suppliers!A31="","",Suppliers!A31)</f>
-        <v/>
-      </c>
-      <c r="B33" s="38" t="str">
-        <f aca="false">IF($A33="","",COUNTIF('Score Log'!$C$4:$C$203,$A33))</f>
-        <v/>
-      </c>
-      <c r="C33" s="39" t="str">
-        <f aca="false">IF($A33="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A33),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D33" s="39" t="str">
-        <f aca="false">IF($A33="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A33),1),"-"))</f>
+      <c r="A33" s="37"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="38" t="str">
+        <f aca="false">IF($B33="","",IF($C33="",COUNTIF('Score Log'!$C$4:$C$203,$B33),COUNTIFS('Score Log'!$C$4:$C$203,$B33,'Score Log'!$D$4:$D$203,$C33)))</f>
         <v/>
       </c>
       <c r="E33" s="39" t="str">
-        <f aca="false">IF($A33="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A33),1),"-"))</f>
+        <f aca="false">IF($B33="","",IFERROR(ROUND(IF($C33="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B33),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B33,'Score Log'!$D$4:$D$203,$C33)),1),"-"))</f>
         <v/>
       </c>
       <c r="F33" s="39" t="str">
-        <f aca="false">IF($A33="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A33),1),"-"))</f>
+        <f aca="false">IF($B33="","",IFERROR(ROUND(IF($C33="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B33),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B33,'Score Log'!$D$4:$D$203,$C33)),1),"-"))</f>
         <v/>
       </c>
       <c r="G33" s="39" t="str">
-        <f aca="false">IF($A33="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A33),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H33" s="40" t="str">
-        <f aca="false">IF($A33="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A33,'Score Log'!$U$4:$U$203,"Yes")/$B33,"-"))</f>
-        <v/>
-      </c>
-      <c r="I33" s="41" t="str">
-        <f aca="false">IF($A33="","",IF(ISNUMBER($D33),MAX(1,MIN(5,ROUND(6-$D33,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J33" s="41" t="str">
-        <f aca="false">IF($A33="","",IF(ISNUMBER($E33),MAX(1,MIN(5,ROUND(6-$E33,0))),"-"))</f>
+        <f aca="false">IF($B33="","",IFERROR(ROUND(IF($C33="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B33),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B33,'Score Log'!$D$4:$D$203,$C33)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H33" s="39" t="str">
+        <f aca="false">IF($B33="","",IFERROR(ROUND(IF($C33="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B33),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B33,'Score Log'!$D$4:$D$203,$C33)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I33" s="39" t="str">
+        <f aca="false">IF($B33="","",IFERROR(ROUND(IF($C33="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B33),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B33,'Score Log'!$D$4:$D$203,$C33)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J33" s="40" t="str">
+        <f aca="false">IF(OR($B33="",$D33=0),"",IFERROR(IF($C33="",COUNTIFS('Score Log'!$C$4:$C$203,$B33,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B33,'Score Log'!$D$4:$D$203,$C33,'Score Log'!$U$4:$U$203,"Yes"))/$D33,"-"))</f>
         <v/>
       </c>
       <c r="K33" s="41" t="str">
-        <f aca="false">IF($A33="","",IF(AND(ISNUMBER($F33),ISNUMBER($C33)),MAX(1,MIN(5,ROUND(6-AVERAGE($F33,$C33),0))),IF(ISNUMBER($F33),MAX(1,MIN(5,ROUND(6-$F33,0))),"-")))</f>
+        <f aca="false">IF($B33="","",IF(ISNUMBER($F33),MAX(1,MIN(5,ROUND(6-$F33,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L33" s="41" t="str">
+        <f aca="false">IF($B33="","",IF(ISNUMBER($G33),MAX(1,MIN(5,ROUND(6-$G33,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M33" s="41" t="str">
+        <f aca="false">IF($B33="","",IF(AND(ISNUMBER($P33),ISNUMBER($O33)),MAX(1,MIN(5,ROUND(6-AVERAGE($P33,$O33),0))),IF(ISNUMBER($P33),MAX(1,MIN(5,ROUND(6-$P33,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O33" s="33" t="str">
+        <f aca="false">IF($B33="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B33),""))</f>
+        <v/>
+      </c>
+      <c r="P33" s="33" t="str">
+        <f aca="false">IF($B33="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B33),""))</f>
         <v/>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="37" t="str">
-        <f aca="false">IF(Suppliers!A32="","",Suppliers!A32)</f>
-        <v/>
-      </c>
-      <c r="B34" s="38" t="str">
-        <f aca="false">IF($A34="","",COUNTIF('Score Log'!$C$4:$C$203,$A34))</f>
-        <v/>
-      </c>
-      <c r="C34" s="39" t="str">
-        <f aca="false">IF($A34="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$A34),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="D34" s="39" t="str">
-        <f aca="false">IF($A34="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$A34),1),"-"))</f>
+      <c r="A34" s="37"/>
+      <c r="B34" s="37"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="38" t="str">
+        <f aca="false">IF($B34="","",IF($C34="",COUNTIF('Score Log'!$C$4:$C$203,$B34),COUNTIFS('Score Log'!$C$4:$C$203,$B34,'Score Log'!$D$4:$D$203,$C34)))</f>
         <v/>
       </c>
       <c r="E34" s="39" t="str">
-        <f aca="false">IF($A34="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$A34),1),"-"))</f>
+        <f aca="false">IF($B34="","",IFERROR(ROUND(IF($C34="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B34),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B34,'Score Log'!$D$4:$D$203,$C34)),1),"-"))</f>
         <v/>
       </c>
       <c r="F34" s="39" t="str">
-        <f aca="false">IF($A34="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$A34),1),"-"))</f>
+        <f aca="false">IF($B34="","",IFERROR(ROUND(IF($C34="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B34),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B34,'Score Log'!$D$4:$D$203,$C34)),1),"-"))</f>
         <v/>
       </c>
       <c r="G34" s="39" t="str">
-        <f aca="false">IF($A34="","",IFERROR(ROUND(AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$A34),1),"-"))</f>
-        <v/>
-      </c>
-      <c r="H34" s="40" t="str">
-        <f aca="false">IF($A34="","",IFERROR(COUNTIFS('Score Log'!$C$4:$C$203,$A34,'Score Log'!$U$4:$U$203,"Yes")/$B34,"-"))</f>
-        <v/>
-      </c>
-      <c r="I34" s="41" t="str">
-        <f aca="false">IF($A34="","",IF(ISNUMBER($D34),MAX(1,MIN(5,ROUND(6-$D34,0))),"-"))</f>
-        <v/>
-      </c>
-      <c r="J34" s="41" t="str">
-        <f aca="false">IF($A34="","",IF(ISNUMBER($E34),MAX(1,MIN(5,ROUND(6-$E34,0))),"-"))</f>
+        <f aca="false">IF($B34="","",IFERROR(ROUND(IF($C34="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B34),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B34,'Score Log'!$D$4:$D$203,$C34)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H34" s="39" t="str">
+        <f aca="false">IF($B34="","",IFERROR(ROUND(IF($C34="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B34),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B34,'Score Log'!$D$4:$D$203,$C34)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I34" s="39" t="str">
+        <f aca="false">IF($B34="","",IFERROR(ROUND(IF($C34="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B34),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B34,'Score Log'!$D$4:$D$203,$C34)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J34" s="40" t="str">
+        <f aca="false">IF(OR($B34="",$D34=0),"",IFERROR(IF($C34="",COUNTIFS('Score Log'!$C$4:$C$203,$B34,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B34,'Score Log'!$D$4:$D$203,$C34,'Score Log'!$U$4:$U$203,"Yes"))/$D34,"-"))</f>
         <v/>
       </c>
       <c r="K34" s="41" t="str">
-        <f aca="false">IF($A34="","",IF(AND(ISNUMBER($F34),ISNUMBER($C34)),MAX(1,MIN(5,ROUND(6-AVERAGE($F34,$C34),0))),IF(ISNUMBER($F34),MAX(1,MIN(5,ROUND(6-$F34,0))),"-")))</f>
+        <f aca="false">IF($B34="","",IF(ISNUMBER($F34),MAX(1,MIN(5,ROUND(6-$F34,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L34" s="41" t="str">
+        <f aca="false">IF($B34="","",IF(ISNUMBER($G34),MAX(1,MIN(5,ROUND(6-$G34,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M34" s="41" t="str">
+        <f aca="false">IF($B34="","",IF(AND(ISNUMBER($P34),ISNUMBER($O34)),MAX(1,MIN(5,ROUND(6-AVERAGE($P34,$O34),0))),IF(ISNUMBER($P34),MAX(1,MIN(5,ROUND(6-$P34,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O34" s="33" t="str">
+        <f aca="false">IF($B34="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B34),""))</f>
+        <v/>
+      </c>
+      <c r="P34" s="33" t="str">
+        <f aca="false">IF($B34="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B34),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="37"/>
+      <c r="B35" s="37"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="38" t="str">
+        <f aca="false">IF($B35="","",IF($C35="",COUNTIF('Score Log'!$C$4:$C$203,$B35),COUNTIFS('Score Log'!$C$4:$C$203,$B35,'Score Log'!$D$4:$D$203,$C35)))</f>
+        <v/>
+      </c>
+      <c r="E35" s="39" t="str">
+        <f aca="false">IF($B35="","",IFERROR(ROUND(IF($C35="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B35),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B35,'Score Log'!$D$4:$D$203,$C35)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="F35" s="39" t="str">
+        <f aca="false">IF($B35="","",IFERROR(ROUND(IF($C35="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B35),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B35,'Score Log'!$D$4:$D$203,$C35)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="G35" s="39" t="str">
+        <f aca="false">IF($B35="","",IFERROR(ROUND(IF($C35="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B35),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B35,'Score Log'!$D$4:$D$203,$C35)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H35" s="39" t="str">
+        <f aca="false">IF($B35="","",IFERROR(ROUND(IF($C35="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B35),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B35,'Score Log'!$D$4:$D$203,$C35)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I35" s="39" t="str">
+        <f aca="false">IF($B35="","",IFERROR(ROUND(IF($C35="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B35),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B35,'Score Log'!$D$4:$D$203,$C35)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J35" s="40" t="str">
+        <f aca="false">IF(OR($B35="",$D35=0),"",IFERROR(IF($C35="",COUNTIFS('Score Log'!$C$4:$C$203,$B35,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B35,'Score Log'!$D$4:$D$203,$C35,'Score Log'!$U$4:$U$203,"Yes"))/$D35,"-"))</f>
+        <v/>
+      </c>
+      <c r="K35" s="41" t="str">
+        <f aca="false">IF($B35="","",IF(ISNUMBER($F35),MAX(1,MIN(5,ROUND(6-$F35,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L35" s="41" t="str">
+        <f aca="false">IF($B35="","",IF(ISNUMBER($G35),MAX(1,MIN(5,ROUND(6-$G35,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M35" s="41" t="str">
+        <f aca="false">IF($B35="","",IF(AND(ISNUMBER($P35),ISNUMBER($O35)),MAX(1,MIN(5,ROUND(6-AVERAGE($P35,$O35),0))),IF(ISNUMBER($P35),MAX(1,MIN(5,ROUND(6-$P35,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O35" s="33" t="str">
+        <f aca="false">IF($B35="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B35),""))</f>
+        <v/>
+      </c>
+      <c r="P35" s="33" t="str">
+        <f aca="false">IF($B35="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B35),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="37"/>
+      <c r="B36" s="37"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="38" t="str">
+        <f aca="false">IF($B36="","",IF($C36="",COUNTIF('Score Log'!$C$4:$C$203,$B36),COUNTIFS('Score Log'!$C$4:$C$203,$B36,'Score Log'!$D$4:$D$203,$C36)))</f>
+        <v/>
+      </c>
+      <c r="E36" s="39" t="str">
+        <f aca="false">IF($B36="","",IFERROR(ROUND(IF($C36="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B36),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B36,'Score Log'!$D$4:$D$203,$C36)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="F36" s="39" t="str">
+        <f aca="false">IF($B36="","",IFERROR(ROUND(IF($C36="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B36),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B36,'Score Log'!$D$4:$D$203,$C36)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="G36" s="39" t="str">
+        <f aca="false">IF($B36="","",IFERROR(ROUND(IF($C36="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B36),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B36,'Score Log'!$D$4:$D$203,$C36)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H36" s="39" t="str">
+        <f aca="false">IF($B36="","",IFERROR(ROUND(IF($C36="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B36),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B36,'Score Log'!$D$4:$D$203,$C36)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I36" s="39" t="str">
+        <f aca="false">IF($B36="","",IFERROR(ROUND(IF($C36="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B36),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B36,'Score Log'!$D$4:$D$203,$C36)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J36" s="40" t="str">
+        <f aca="false">IF(OR($B36="",$D36=0),"",IFERROR(IF($C36="",COUNTIFS('Score Log'!$C$4:$C$203,$B36,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B36,'Score Log'!$D$4:$D$203,$C36,'Score Log'!$U$4:$U$203,"Yes"))/$D36,"-"))</f>
+        <v/>
+      </c>
+      <c r="K36" s="41" t="str">
+        <f aca="false">IF($B36="","",IF(ISNUMBER($F36),MAX(1,MIN(5,ROUND(6-$F36,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L36" s="41" t="str">
+        <f aca="false">IF($B36="","",IF(ISNUMBER($G36),MAX(1,MIN(5,ROUND(6-$G36,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M36" s="41" t="str">
+        <f aca="false">IF($B36="","",IF(AND(ISNUMBER($P36),ISNUMBER($O36)),MAX(1,MIN(5,ROUND(6-AVERAGE($P36,$O36),0))),IF(ISNUMBER($P36),MAX(1,MIN(5,ROUND(6-$P36,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O36" s="33" t="str">
+        <f aca="false">IF($B36="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B36),""))</f>
+        <v/>
+      </c>
+      <c r="P36" s="33" t="str">
+        <f aca="false">IF($B36="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B36),""))</f>
         <v/>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="42" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="43" t="s">
-        <v>83</v>
-      </c>
-      <c r="B38" s="43"/>
-      <c r="C38" s="43"/>
-      <c r="D38" s="43"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="43"/>
-      <c r="G38" s="43"/>
-      <c r="H38" s="43"/>
-      <c r="I38" s="43"/>
-      <c r="J38" s="43"/>
-      <c r="K38" s="43"/>
-    </row>
-    <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="43" t="s">
-        <v>84</v>
-      </c>
-      <c r="B39" s="43"/>
-      <c r="C39" s="43"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="43"/>
-      <c r="I39" s="43"/>
-      <c r="J39" s="43"/>
-      <c r="K39" s="43"/>
-    </row>
-    <row r="40" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="43" t="s">
-        <v>85</v>
-      </c>
-      <c r="B40" s="43"/>
-      <c r="C40" s="43"/>
-      <c r="D40" s="43"/>
-      <c r="E40" s="43"/>
-      <c r="F40" s="43"/>
-      <c r="G40" s="43"/>
-      <c r="H40" s="43"/>
-      <c r="I40" s="43"/>
-      <c r="J40" s="43"/>
-      <c r="K40" s="43"/>
-    </row>
-    <row r="41" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="43" t="s">
+      <c r="A37" s="37"/>
+      <c r="B37" s="37"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="38" t="str">
+        <f aca="false">IF($B37="","",IF($C37="",COUNTIF('Score Log'!$C$4:$C$203,$B37),COUNTIFS('Score Log'!$C$4:$C$203,$B37,'Score Log'!$D$4:$D$203,$C37)))</f>
+        <v/>
+      </c>
+      <c r="E37" s="39" t="str">
+        <f aca="false">IF($B37="","",IFERROR(ROUND(IF($C37="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B37),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B37,'Score Log'!$D$4:$D$203,$C37)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="F37" s="39" t="str">
+        <f aca="false">IF($B37="","",IFERROR(ROUND(IF($C37="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B37),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B37,'Score Log'!$D$4:$D$203,$C37)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="G37" s="39" t="str">
+        <f aca="false">IF($B37="","",IFERROR(ROUND(IF($C37="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B37),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B37,'Score Log'!$D$4:$D$203,$C37)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H37" s="39" t="str">
+        <f aca="false">IF($B37="","",IFERROR(ROUND(IF($C37="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B37),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B37,'Score Log'!$D$4:$D$203,$C37)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I37" s="39" t="str">
+        <f aca="false">IF($B37="","",IFERROR(ROUND(IF($C37="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B37),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B37,'Score Log'!$D$4:$D$203,$C37)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J37" s="40" t="str">
+        <f aca="false">IF(OR($B37="",$D37=0),"",IFERROR(IF($C37="",COUNTIFS('Score Log'!$C$4:$C$203,$B37,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B37,'Score Log'!$D$4:$D$203,$C37,'Score Log'!$U$4:$U$203,"Yes"))/$D37,"-"))</f>
+        <v/>
+      </c>
+      <c r="K37" s="41" t="str">
+        <f aca="false">IF($B37="","",IF(ISNUMBER($F37),MAX(1,MIN(5,ROUND(6-$F37,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L37" s="41" t="str">
+        <f aca="false">IF($B37="","",IF(ISNUMBER($G37),MAX(1,MIN(5,ROUND(6-$G37,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M37" s="41" t="str">
+        <f aca="false">IF($B37="","",IF(AND(ISNUMBER($P37),ISNUMBER($O37)),MAX(1,MIN(5,ROUND(6-AVERAGE($P37,$O37),0))),IF(ISNUMBER($P37),MAX(1,MIN(5,ROUND(6-$P37,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O37" s="33" t="str">
+        <f aca="false">IF($B37="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B37),""))</f>
+        <v/>
+      </c>
+      <c r="P37" s="33" t="str">
+        <f aca="false">IF($B37="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B37),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="37"/>
+      <c r="B38" s="37"/>
+      <c r="C38" s="37"/>
+      <c r="D38" s="38" t="str">
+        <f aca="false">IF($B38="","",IF($C38="",COUNTIF('Score Log'!$C$4:$C$203,$B38),COUNTIFS('Score Log'!$C$4:$C$203,$B38,'Score Log'!$D$4:$D$203,$C38)))</f>
+        <v/>
+      </c>
+      <c r="E38" s="39" t="str">
+        <f aca="false">IF($B38="","",IFERROR(ROUND(IF($C38="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B38),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B38,'Score Log'!$D$4:$D$203,$C38)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="F38" s="39" t="str">
+        <f aca="false">IF($B38="","",IFERROR(ROUND(IF($C38="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B38),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B38,'Score Log'!$D$4:$D$203,$C38)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="G38" s="39" t="str">
+        <f aca="false">IF($B38="","",IFERROR(ROUND(IF($C38="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B38),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B38,'Score Log'!$D$4:$D$203,$C38)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H38" s="39" t="str">
+        <f aca="false">IF($B38="","",IFERROR(ROUND(IF($C38="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B38),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B38,'Score Log'!$D$4:$D$203,$C38)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I38" s="39" t="str">
+        <f aca="false">IF($B38="","",IFERROR(ROUND(IF($C38="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B38),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B38,'Score Log'!$D$4:$D$203,$C38)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J38" s="40" t="str">
+        <f aca="false">IF(OR($B38="",$D38=0),"",IFERROR(IF($C38="",COUNTIFS('Score Log'!$C$4:$C$203,$B38,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B38,'Score Log'!$D$4:$D$203,$C38,'Score Log'!$U$4:$U$203,"Yes"))/$D38,"-"))</f>
+        <v/>
+      </c>
+      <c r="K38" s="41" t="str">
+        <f aca="false">IF($B38="","",IF(ISNUMBER($F38),MAX(1,MIN(5,ROUND(6-$F38,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L38" s="41" t="str">
+        <f aca="false">IF($B38="","",IF(ISNUMBER($G38),MAX(1,MIN(5,ROUND(6-$G38,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M38" s="41" t="str">
+        <f aca="false">IF($B38="","",IF(AND(ISNUMBER($P38),ISNUMBER($O38)),MAX(1,MIN(5,ROUND(6-AVERAGE($P38,$O38),0))),IF(ISNUMBER($P38),MAX(1,MIN(5,ROUND(6-$P38,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O38" s="33" t="str">
+        <f aca="false">IF($B38="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B38),""))</f>
+        <v/>
+      </c>
+      <c r="P38" s="33" t="str">
+        <f aca="false">IF($B38="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B38),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="37"/>
+      <c r="B39" s="37"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="38" t="str">
+        <f aca="false">IF($B39="","",IF($C39="",COUNTIF('Score Log'!$C$4:$C$203,$B39),COUNTIFS('Score Log'!$C$4:$C$203,$B39,'Score Log'!$D$4:$D$203,$C39)))</f>
+        <v/>
+      </c>
+      <c r="E39" s="39" t="str">
+        <f aca="false">IF($B39="","",IFERROR(ROUND(IF($C39="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B39),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B39,'Score Log'!$D$4:$D$203,$C39)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="F39" s="39" t="str">
+        <f aca="false">IF($B39="","",IFERROR(ROUND(IF($C39="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B39),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B39,'Score Log'!$D$4:$D$203,$C39)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="G39" s="39" t="str">
+        <f aca="false">IF($B39="","",IFERROR(ROUND(IF($C39="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B39),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B39,'Score Log'!$D$4:$D$203,$C39)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H39" s="39" t="str">
+        <f aca="false">IF($B39="","",IFERROR(ROUND(IF($C39="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B39),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B39,'Score Log'!$D$4:$D$203,$C39)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I39" s="39" t="str">
+        <f aca="false">IF($B39="","",IFERROR(ROUND(IF($C39="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B39),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B39,'Score Log'!$D$4:$D$203,$C39)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J39" s="40" t="str">
+        <f aca="false">IF(OR($B39="",$D39=0),"",IFERROR(IF($C39="",COUNTIFS('Score Log'!$C$4:$C$203,$B39,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B39,'Score Log'!$D$4:$D$203,$C39,'Score Log'!$U$4:$U$203,"Yes"))/$D39,"-"))</f>
+        <v/>
+      </c>
+      <c r="K39" s="41" t="str">
+        <f aca="false">IF($B39="","",IF(ISNUMBER($F39),MAX(1,MIN(5,ROUND(6-$F39,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L39" s="41" t="str">
+        <f aca="false">IF($B39="","",IF(ISNUMBER($G39),MAX(1,MIN(5,ROUND(6-$G39,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M39" s="41" t="str">
+        <f aca="false">IF($B39="","",IF(AND(ISNUMBER($P39),ISNUMBER($O39)),MAX(1,MIN(5,ROUND(6-AVERAGE($P39,$O39),0))),IF(ISNUMBER($P39),MAX(1,MIN(5,ROUND(6-$P39,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O39" s="33" t="str">
+        <f aca="false">IF($B39="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B39),""))</f>
+        <v/>
+      </c>
+      <c r="P39" s="33" t="str">
+        <f aca="false">IF($B39="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B39),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="37"/>
+      <c r="B40" s="37"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="38" t="str">
+        <f aca="false">IF($B40="","",IF($C40="",COUNTIF('Score Log'!$C$4:$C$203,$B40),COUNTIFS('Score Log'!$C$4:$C$203,$B40,'Score Log'!$D$4:$D$203,$C40)))</f>
+        <v/>
+      </c>
+      <c r="E40" s="39" t="str">
+        <f aca="false">IF($B40="","",IFERROR(ROUND(IF($C40="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B40),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B40,'Score Log'!$D$4:$D$203,$C40)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="F40" s="39" t="str">
+        <f aca="false">IF($B40="","",IFERROR(ROUND(IF($C40="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B40),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B40,'Score Log'!$D$4:$D$203,$C40)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="G40" s="39" t="str">
+        <f aca="false">IF($B40="","",IFERROR(ROUND(IF($C40="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B40),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B40,'Score Log'!$D$4:$D$203,$C40)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H40" s="39" t="str">
+        <f aca="false">IF($B40="","",IFERROR(ROUND(IF($C40="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B40),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B40,'Score Log'!$D$4:$D$203,$C40)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I40" s="39" t="str">
+        <f aca="false">IF($B40="","",IFERROR(ROUND(IF($C40="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B40),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B40,'Score Log'!$D$4:$D$203,$C40)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J40" s="40" t="str">
+        <f aca="false">IF(OR($B40="",$D40=0),"",IFERROR(IF($C40="",COUNTIFS('Score Log'!$C$4:$C$203,$B40,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B40,'Score Log'!$D$4:$D$203,$C40,'Score Log'!$U$4:$U$203,"Yes"))/$D40,"-"))</f>
+        <v/>
+      </c>
+      <c r="K40" s="41" t="str">
+        <f aca="false">IF($B40="","",IF(ISNUMBER($F40),MAX(1,MIN(5,ROUND(6-$F40,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L40" s="41" t="str">
+        <f aca="false">IF($B40="","",IF(ISNUMBER($G40),MAX(1,MIN(5,ROUND(6-$G40,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M40" s="41" t="str">
+        <f aca="false">IF($B40="","",IF(AND(ISNUMBER($P40),ISNUMBER($O40)),MAX(1,MIN(5,ROUND(6-AVERAGE($P40,$O40),0))),IF(ISNUMBER($P40),MAX(1,MIN(5,ROUND(6-$P40,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O40" s="33" t="str">
+        <f aca="false">IF($B40="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B40),""))</f>
+        <v/>
+      </c>
+      <c r="P40" s="33" t="str">
+        <f aca="false">IF($B40="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B40),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="37"/>
+      <c r="B41" s="37"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="38" t="str">
+        <f aca="false">IF($B41="","",IF($C41="",COUNTIF('Score Log'!$C$4:$C$203,$B41),COUNTIFS('Score Log'!$C$4:$C$203,$B41,'Score Log'!$D$4:$D$203,$C41)))</f>
+        <v/>
+      </c>
+      <c r="E41" s="39" t="str">
+        <f aca="false">IF($B41="","",IFERROR(ROUND(IF($C41="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B41),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B41,'Score Log'!$D$4:$D$203,$C41)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="F41" s="39" t="str">
+        <f aca="false">IF($B41="","",IFERROR(ROUND(IF($C41="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B41),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B41,'Score Log'!$D$4:$D$203,$C41)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="G41" s="39" t="str">
+        <f aca="false">IF($B41="","",IFERROR(ROUND(IF($C41="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B41),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B41,'Score Log'!$D$4:$D$203,$C41)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H41" s="39" t="str">
+        <f aca="false">IF($B41="","",IFERROR(ROUND(IF($C41="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B41),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B41,'Score Log'!$D$4:$D$203,$C41)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I41" s="39" t="str">
+        <f aca="false">IF($B41="","",IFERROR(ROUND(IF($C41="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B41),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B41,'Score Log'!$D$4:$D$203,$C41)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J41" s="40" t="str">
+        <f aca="false">IF(OR($B41="",$D41=0),"",IFERROR(IF($C41="",COUNTIFS('Score Log'!$C$4:$C$203,$B41,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B41,'Score Log'!$D$4:$D$203,$C41,'Score Log'!$U$4:$U$203,"Yes"))/$D41,"-"))</f>
+        <v/>
+      </c>
+      <c r="K41" s="41" t="str">
+        <f aca="false">IF($B41="","",IF(ISNUMBER($F41),MAX(1,MIN(5,ROUND(6-$F41,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L41" s="41" t="str">
+        <f aca="false">IF($B41="","",IF(ISNUMBER($G41),MAX(1,MIN(5,ROUND(6-$G41,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M41" s="41" t="str">
+        <f aca="false">IF($B41="","",IF(AND(ISNUMBER($P41),ISNUMBER($O41)),MAX(1,MIN(5,ROUND(6-AVERAGE($P41,$O41),0))),IF(ISNUMBER($P41),MAX(1,MIN(5,ROUND(6-$P41,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O41" s="33" t="str">
+        <f aca="false">IF($B41="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B41),""))</f>
+        <v/>
+      </c>
+      <c r="P41" s="33" t="str">
+        <f aca="false">IF($B41="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B41),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="37"/>
+      <c r="B42" s="37"/>
+      <c r="C42" s="37"/>
+      <c r="D42" s="38" t="str">
+        <f aca="false">IF($B42="","",IF($C42="",COUNTIF('Score Log'!$C$4:$C$203,$B42),COUNTIFS('Score Log'!$C$4:$C$203,$B42,'Score Log'!$D$4:$D$203,$C42)))</f>
+        <v/>
+      </c>
+      <c r="E42" s="39" t="str">
+        <f aca="false">IF($B42="","",IFERROR(ROUND(IF($C42="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B42),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B42,'Score Log'!$D$4:$D$203,$C42)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="F42" s="39" t="str">
+        <f aca="false">IF($B42="","",IFERROR(ROUND(IF($C42="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B42),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B42,'Score Log'!$D$4:$D$203,$C42)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="G42" s="39" t="str">
+        <f aca="false">IF($B42="","",IFERROR(ROUND(IF($C42="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B42),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B42,'Score Log'!$D$4:$D$203,$C42)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H42" s="39" t="str">
+        <f aca="false">IF($B42="","",IFERROR(ROUND(IF($C42="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B42),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B42,'Score Log'!$D$4:$D$203,$C42)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I42" s="39" t="str">
+        <f aca="false">IF($B42="","",IFERROR(ROUND(IF($C42="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B42),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B42,'Score Log'!$D$4:$D$203,$C42)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J42" s="40" t="str">
+        <f aca="false">IF(OR($B42="",$D42=0),"",IFERROR(IF($C42="",COUNTIFS('Score Log'!$C$4:$C$203,$B42,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B42,'Score Log'!$D$4:$D$203,$C42,'Score Log'!$U$4:$U$203,"Yes"))/$D42,"-"))</f>
+        <v/>
+      </c>
+      <c r="K42" s="41" t="str">
+        <f aca="false">IF($B42="","",IF(ISNUMBER($F42),MAX(1,MIN(5,ROUND(6-$F42,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L42" s="41" t="str">
+        <f aca="false">IF($B42="","",IF(ISNUMBER($G42),MAX(1,MIN(5,ROUND(6-$G42,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M42" s="41" t="str">
+        <f aca="false">IF($B42="","",IF(AND(ISNUMBER($P42),ISNUMBER($O42)),MAX(1,MIN(5,ROUND(6-AVERAGE($P42,$O42),0))),IF(ISNUMBER($P42),MAX(1,MIN(5,ROUND(6-$P42,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O42" s="33" t="str">
+        <f aca="false">IF($B42="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B42),""))</f>
+        <v/>
+      </c>
+      <c r="P42" s="33" t="str">
+        <f aca="false">IF($B42="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B42),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="37"/>
+      <c r="B43" s="37"/>
+      <c r="C43" s="37"/>
+      <c r="D43" s="38" t="str">
+        <f aca="false">IF($B43="","",IF($C43="",COUNTIF('Score Log'!$C$4:$C$203,$B43),COUNTIFS('Score Log'!$C$4:$C$203,$B43,'Score Log'!$D$4:$D$203,$C43)))</f>
+        <v/>
+      </c>
+      <c r="E43" s="39" t="str">
+        <f aca="false">IF($B43="","",IFERROR(ROUND(IF($C43="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B43),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B43,'Score Log'!$D$4:$D$203,$C43)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="F43" s="39" t="str">
+        <f aca="false">IF($B43="","",IFERROR(ROUND(IF($C43="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B43),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B43,'Score Log'!$D$4:$D$203,$C43)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="G43" s="39" t="str">
+        <f aca="false">IF($B43="","",IFERROR(ROUND(IF($C43="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B43),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B43,'Score Log'!$D$4:$D$203,$C43)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H43" s="39" t="str">
+        <f aca="false">IF($B43="","",IFERROR(ROUND(IF($C43="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B43),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B43,'Score Log'!$D$4:$D$203,$C43)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I43" s="39" t="str">
+        <f aca="false">IF($B43="","",IFERROR(ROUND(IF($C43="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B43),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B43,'Score Log'!$D$4:$D$203,$C43)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J43" s="40" t="str">
+        <f aca="false">IF(OR($B43="",$D43=0),"",IFERROR(IF($C43="",COUNTIFS('Score Log'!$C$4:$C$203,$B43,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B43,'Score Log'!$D$4:$D$203,$C43,'Score Log'!$U$4:$U$203,"Yes"))/$D43,"-"))</f>
+        <v/>
+      </c>
+      <c r="K43" s="41" t="str">
+        <f aca="false">IF($B43="","",IF(ISNUMBER($F43),MAX(1,MIN(5,ROUND(6-$F43,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L43" s="41" t="str">
+        <f aca="false">IF($B43="","",IF(ISNUMBER($G43),MAX(1,MIN(5,ROUND(6-$G43,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M43" s="41" t="str">
+        <f aca="false">IF($B43="","",IF(AND(ISNUMBER($P43),ISNUMBER($O43)),MAX(1,MIN(5,ROUND(6-AVERAGE($P43,$O43),0))),IF(ISNUMBER($P43),MAX(1,MIN(5,ROUND(6-$P43,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O43" s="33" t="str">
+        <f aca="false">IF($B43="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B43),""))</f>
+        <v/>
+      </c>
+      <c r="P43" s="33" t="str">
+        <f aca="false">IF($B43="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B43),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="37"/>
+      <c r="B44" s="37"/>
+      <c r="C44" s="37"/>
+      <c r="D44" s="38" t="str">
+        <f aca="false">IF($B44="","",IF($C44="",COUNTIF('Score Log'!$C$4:$C$203,$B44),COUNTIFS('Score Log'!$C$4:$C$203,$B44,'Score Log'!$D$4:$D$203,$C44)))</f>
+        <v/>
+      </c>
+      <c r="E44" s="39" t="str">
+        <f aca="false">IF($B44="","",IFERROR(ROUND(IF($C44="",AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B44),AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B44,'Score Log'!$D$4:$D$203,$C44)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="F44" s="39" t="str">
+        <f aca="false">IF($B44="","",IFERROR(ROUND(IF($C44="",AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B44),AVERAGEIFS('Score Log'!$H$4:$H$203,'Score Log'!$C$4:$C$203,$B44,'Score Log'!$D$4:$D$203,$C44)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="G44" s="39" t="str">
+        <f aca="false">IF($B44="","",IFERROR(ROUND(IF($C44="",AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B44),AVERAGEIFS('Score Log'!$J$4:$J$203,'Score Log'!$C$4:$C$203,$B44,'Score Log'!$D$4:$D$203,$C44)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="H44" s="39" t="str">
+        <f aca="false">IF($B44="","",IFERROR(ROUND(IF($C44="",AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B44),AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B44,'Score Log'!$D$4:$D$203,$C44)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="I44" s="39" t="str">
+        <f aca="false">IF($B44="","",IFERROR(ROUND(IF($C44="",AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B44),AVERAGEIFS('Score Log'!$N$4:$N$203,'Score Log'!$C$4:$C$203,$B44,'Score Log'!$D$4:$D$203,$C44)),1),"-"))</f>
+        <v/>
+      </c>
+      <c r="J44" s="40" t="str">
+        <f aca="false">IF(OR($B44="",$D44=0),"",IFERROR(IF($C44="",COUNTIFS('Score Log'!$C$4:$C$203,$B44,'Score Log'!$U$4:$U$203,"Yes"),COUNTIFS('Score Log'!$C$4:$C$203,$B44,'Score Log'!$D$4:$D$203,$C44,'Score Log'!$U$4:$U$203,"Yes"))/$D44,"-"))</f>
+        <v/>
+      </c>
+      <c r="K44" s="41" t="str">
+        <f aca="false">IF($B44="","",IF(ISNUMBER($F44),MAX(1,MIN(5,ROUND(6-$F44,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="L44" s="41" t="str">
+        <f aca="false">IF($B44="","",IF(ISNUMBER($G44),MAX(1,MIN(5,ROUND(6-$G44,0))),"-"))</f>
+        <v/>
+      </c>
+      <c r="M44" s="41" t="str">
+        <f aca="false">IF($B44="","",IF(AND(ISNUMBER($P44),ISNUMBER($O44)),MAX(1,MIN(5,ROUND(6-AVERAGE($P44,$O44),0))),IF(ISNUMBER($P44),MAX(1,MIN(5,ROUND(6-$P44,0))),"-")))</f>
+        <v/>
+      </c>
+      <c r="O44" s="33" t="str">
+        <f aca="false">IF($B44="","",IFERROR(AVERAGEIFS('Score Log'!$F$4:$F$203,'Score Log'!$C$4:$C$203,$B44),""))</f>
+        <v/>
+      </c>
+      <c r="P44" s="33" t="str">
+        <f aca="false">IF($B44="","",IFERROR(AVERAGEIFS('Score Log'!$L$4:$L$203,'Score Log'!$C$4:$C$203,$B44),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B41" s="43"/>
-      <c r="C41" s="43"/>
-      <c r="D41" s="43"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="43"/>
-      <c r="G41" s="43"/>
-      <c r="H41" s="43"/>
-      <c r="I41" s="43"/>
-      <c r="J41" s="43"/>
-      <c r="K41" s="43"/>
-    </row>
-    <row r="42" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="43" t="s">
+    </row>
+    <row r="48" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="43" t="s">
         <v>87</v>
       </c>
-      <c r="B42" s="43"/>
-      <c r="C42" s="43"/>
-      <c r="D42" s="43"/>
-      <c r="E42" s="43"/>
-      <c r="F42" s="43"/>
-      <c r="G42" s="43"/>
-      <c r="H42" s="43"/>
-      <c r="I42" s="43"/>
-      <c r="J42" s="43"/>
-      <c r="K42" s="43"/>
+      <c r="B48" s="43"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="43"/>
+      <c r="I48" s="43"/>
+      <c r="J48" s="43"/>
+      <c r="K48" s="43"/>
+      <c r="L48" s="43"/>
+      <c r="M48" s="43"/>
+    </row>
+    <row r="49" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="43" t="s">
+        <v>88</v>
+      </c>
+      <c r="B49" s="43"/>
+      <c r="C49" s="43"/>
+      <c r="D49" s="43"/>
+      <c r="E49" s="43"/>
+      <c r="F49" s="43"/>
+      <c r="G49" s="43"/>
+      <c r="H49" s="43"/>
+      <c r="I49" s="43"/>
+      <c r="J49" s="43"/>
+      <c r="K49" s="43"/>
+      <c r="L49" s="43"/>
+      <c r="M49" s="43"/>
+    </row>
+    <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="43" t="s">
+        <v>89</v>
+      </c>
+      <c r="B50" s="43"/>
+      <c r="C50" s="43"/>
+      <c r="D50" s="43"/>
+      <c r="E50" s="43"/>
+      <c r="F50" s="43"/>
+      <c r="G50" s="43"/>
+      <c r="H50" s="43"/>
+      <c r="I50" s="43"/>
+      <c r="J50" s="43"/>
+      <c r="K50" s="43"/>
+      <c r="L50" s="43"/>
+      <c r="M50" s="43"/>
+    </row>
+    <row r="51" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="43" t="s">
+        <v>90</v>
+      </c>
+      <c r="B51" s="43"/>
+      <c r="C51" s="43"/>
+      <c r="D51" s="43"/>
+      <c r="E51" s="43"/>
+      <c r="F51" s="43"/>
+      <c r="G51" s="43"/>
+      <c r="H51" s="43"/>
+      <c r="I51" s="43"/>
+      <c r="J51" s="43"/>
+      <c r="K51" s="43"/>
+      <c r="L51" s="43"/>
+      <c r="M51" s="43"/>
+    </row>
+    <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="43" t="s">
+        <v>91</v>
+      </c>
+      <c r="B52" s="43"/>
+      <c r="C52" s="43"/>
+      <c r="D52" s="43"/>
+      <c r="E52" s="43"/>
+      <c r="F52" s="43"/>
+      <c r="G52" s="43"/>
+      <c r="H52" s="43"/>
+      <c r="I52" s="43"/>
+      <c r="J52" s="43"/>
+      <c r="K52" s="43"/>
+      <c r="L52" s="43"/>
+      <c r="M52" s="43"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="A38:K38"/>
-    <mergeCell ref="A39:K39"/>
-    <mergeCell ref="A40:K40"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A42:K42"/>
+  <mergeCells count="8">
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:J3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="A48:M48"/>
+    <mergeCell ref="A49:M49"/>
+    <mergeCell ref="A50:M50"/>
+    <mergeCell ref="A51:M51"/>
+    <mergeCell ref="A52:M52"/>
   </mergeCells>
-  <conditionalFormatting sqref="C5:G34">
+  <conditionalFormatting sqref="E5:I44">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="1"/>
@@ -13281,7 +14069,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:K34">
+  <conditionalFormatting sqref="K5:M44">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="1"/>
@@ -13293,6 +14081,16 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" error="Pick a supplier from the Suppliers tab (or add it there first)." errorStyle="stop" errorTitle="Unknown supplier" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
+      <formula1>ScorecardSuppliers</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Pick a process from the list in Settings (or add it there first)." errorStyle="stop" errorTitle="Unknown process" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C44" type="list">
+      <formula1>ScorecardProcesses</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -13321,30 +14119,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="44" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C2" s="44" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D2" s="44" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="E2" s="44" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F2" s="44" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13353,13 +14151,13 @@
       </c>
       <c r="B3" s="45"/>
       <c r="C3" s="45" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D3" s="46" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E3" s="45" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F3" s="45"/>
     </row>
@@ -13626,112 +14424,112 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="44" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="F4" s="44" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="48" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B5" s="49" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C5" s="49" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D5" s="49" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="F5" s="49" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="48" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B6" s="49" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C6" s="49" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D6" s="49" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="E6" s="49" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="F6" s="49" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="48" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B7" s="49" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C7" s="49" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D7" s="49" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="E7" s="49" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="F7" s="49" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="48" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B8" s="49" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C8" s="49" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D8" s="49" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E8" s="49" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F8" s="49" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -13762,23 +14560,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="25" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D3" s="25" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="50" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B4" s="51" t="n">
         <v>0.25</v>
@@ -13789,7 +14587,7 @@
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="50" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B5" s="51" t="n">
         <v>0.3</v>
@@ -13800,76 +14598,76 @@
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="50" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B6" s="51" t="n">
         <v>0.25</v>
       </c>
       <c r="D6" s="52" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="50" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B7" s="51" t="n">
         <v>0.2</v>
       </c>
       <c r="D7" s="52" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B8" s="54" t="n">
         <f aca="false">SUM(B4:B7)</f>
         <v>1</v>
       </c>
       <c r="D8" s="52" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D9" s="52" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D10" s="52" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D11" s="52" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D12" s="52" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D13" s="52" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D14" s="52" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D15" s="52" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D16" s="52" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>